<commit_message>
Add feedback workflow and refresh song catalog
</commit_message>
<xml_diff>
--- a/producers/P主代表曲统计表(1).xlsx
+++ b/producers/P主代表曲统计表(1).xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R11c7f12bdb0645bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R278c2299da03444f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1408,6 +1408,9 @@
     <x:t xml:space="preserve">∞ TIMEs</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">我唱人间</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">Lanber</x:t>
   </x:si>
   <x:si>
@@ -1981,16 +1984,19 @@
     <x:r>
       <x:rPr>
         <x:b/>
-        <x:sz val="1400"/>
+        <x:sz val="409"/>
         <x:color rgb="FF000000"/>
+        <x:rFont val="宋体"/>
+        <x:family val="3"/>
       </x:rPr>
       <x:t xml:space="preserve">著小生</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1200"/>
+        <x:sz val="409"/>
         <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
+        <x:family val="2"/>
       </x:rPr>
       <x:t xml:space="preserve">zoki</x:t>
     </x:r>
@@ -2080,48 +2086,55 @@
     <x:r>
       <x:rPr>
         <x:b/>
-        <x:sz val="1400"/>
+        <x:sz val="409"/>
         <x:color rgb="FF000000"/>
+        <x:rFont val="宋体"/>
+        <x:family val="3"/>
       </x:rPr>
       <x:t xml:space="preserve">ChiliChill</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1000"/>
+        <x:sz val="409"/>
         <x:color rgb="FF000000"/>
         <x:rFont val="宋体"/>
+        <x:family val="3"/>
       </x:rPr>
       <x:t xml:space="preserve">（</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1000"/>
+        <x:sz val="409"/>
         <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
+        <x:family val="2"/>
       </x:rPr>
       <x:t xml:space="preserve">Yu.H</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1000"/>
+        <x:sz val="409"/>
         <x:color rgb="FF000000"/>
         <x:rFont val="宋体"/>
+        <x:family val="3"/>
       </x:rPr>
       <x:t xml:space="preserve">、</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1000"/>
+        <x:sz val="409"/>
         <x:color rgb="FF000000"/>
         <x:rFont val="Arial"/>
+        <x:family val="2"/>
       </x:rPr>
       <x:t xml:space="preserve">CuSummer</x:t>
     </x:r>
     <x:r>
       <x:rPr>
-        <x:sz val="1000"/>
+        <x:sz val="409"/>
         <x:color rgb="FF000000"/>
         <x:rFont val="宋体"/>
+        <x:family val="3"/>
       </x:rPr>
       <x:t xml:space="preserve">）</x:t>
     </x:r>
@@ -2151,13 +2164,13 @@
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="6">
     <x:numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <x:numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <x:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <x:numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <x:numFmt numFmtId="176" formatCode="yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;;@"/>
-    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="176" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <x:numFmt numFmtId="177" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <x:numFmt numFmtId="178" formatCode="yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;;@"/>
+    <x:numFmt numFmtId="179" formatCode="yyyy\-mm\-dd"/>
   </x:numFmts>
-  <x:fonts count="27">
+  <x:fonts count="30">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -2290,22 +2303,38 @@
       <x:name val="宋体"/>
     </x:font>
     <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF101418"/>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
       <x:name val="宋体"/>
     </x:font>
     <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF101418"/>
+      <x:b/>
+      <x:sz val="409"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="宋体"/>
+    </x:font>
+    <x:font>
+      <x:sz val="409"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Arial"/>
     </x:font>
     <x:font>
-      <x:sz val="12"/>
-      <x:color rgb="FF101418"/>
-      <x:name val="Arial"/>
+      <x:sz val="409"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="宋体"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:name val="宋体"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="28"/>
+      <x:color theme="4"/>
+      <x:name val="宋体"/>
     </x:font>
   </x:fonts>
-  <x:fills count="33">
+  <x:fills count="34">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2354,12 +2383,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="4" tint="0.79998"/>
+        <x:fgColor theme="4" tint="0.79995"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="4" tint="0.59999"/>
+        <x:fgColor theme="4" tint="0.59996"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -2374,12 +2403,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="5" tint="0.79998"/>
+        <x:fgColor theme="5" tint="0.79995"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="5" tint="0.59999"/>
+        <x:fgColor theme="5" tint="0.59996"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -2394,12 +2423,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="6" tint="0.79998"/>
+        <x:fgColor theme="6" tint="0.79995"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="6" tint="0.59999"/>
+        <x:fgColor theme="6" tint="0.59996"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -2414,12 +2443,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="7" tint="0.79998"/>
+        <x:fgColor theme="7" tint="0.79995"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="7" tint="0.59999"/>
+        <x:fgColor theme="7" tint="0.59996"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -2434,12 +2463,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="8" tint="0.79998"/>
+        <x:fgColor theme="8" tint="0.79995"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="8" tint="0.59999"/>
+        <x:fgColor theme="8" tint="0.59996"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -2454,17 +2483,22 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="9" tint="0.79998"/>
+        <x:fgColor theme="9" tint="0.79995"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="9" tint="0.59999"/>
+        <x:fgColor theme="9" tint="0.59996"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor theme="9" tint="0.39998"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor theme="4" tint="0.39995"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -2491,7 +2525,7 @@
     </x:border>
     <x:border>
       <x:bottom style="medium">
-        <x:color theme="4" tint="0.49998"/>
+        <x:color theme="4" tint="0.49995"/>
       </x:bottom>
     </x:border>
     <x:border>
@@ -2550,23 +2584,23 @@
       </x:bottom>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="49">
+  <x:cellStyleXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <x:xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <x:xf numFmtId="177" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <x:xf numFmtId="9" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <x:xf numFmtId="41" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <x:xf numFmtId="176" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2575,7 +2609,7 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <x:xf numFmtId="0" fontId="24" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2698,6 +2732,9 @@
     <x:xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="33" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellStyleXfs>
   <x:cellXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
@@ -2706,19 +2743,13 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="25" applyFont="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="25" applyFont="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="176" fontId="1" fillId="2" borderId="0" xfId="25" applyNumberFormat="1" applyFont="1">
+    <x:xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <x:xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -2727,246 +2758,75 @@
     <x:xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="179" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="25" applyFont="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="178" fontId="29" fillId="2" borderId="0" xfId="25" applyNumberFormat="1" applyFont="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
-  <x:cellStyles count="49">
-    <x:cellStyle name="常规" xfId="0"/>
-    <x:cellStyle name="千位分隔" xfId="1"/>
-    <x:cellStyle name="货币" xfId="2"/>
+  <x:cellStyles count="50">
+    <x:cellStyle name="20% - 强调文字颜色 1" xfId="26"/>
+    <x:cellStyle name="20% - 强调文字颜色 2" xfId="30"/>
+    <x:cellStyle name="20% - 强调文字颜色 3" xfId="34"/>
+    <x:cellStyle name="20% - 强调文字颜色 4" xfId="38"/>
+    <x:cellStyle name="20% - 强调文字颜色 5" xfId="42"/>
+    <x:cellStyle name="20% - 强调文字颜色 6" xfId="46"/>
+    <x:cellStyle name="40% - 强调文字颜色 1" xfId="27"/>
+    <x:cellStyle name="40% - 强调文字颜色 2" xfId="31"/>
+    <x:cellStyle name="40% - 强调文字颜色 3" xfId="35"/>
+    <x:cellStyle name="40% - 强调文字颜色 4" xfId="39"/>
+    <x:cellStyle name="40% - 强调文字颜色 5" xfId="43"/>
+    <x:cellStyle name="40% - 强调文字颜色 6" xfId="47"/>
+    <x:cellStyle name="60% - 强调文字颜色 1" xfId="28"/>
+    <x:cellStyle name="60% - 强调文字颜色 2" xfId="32"/>
+    <x:cellStyle name="60% - 强调文字颜色 3" xfId="36"/>
+    <x:cellStyle name="60% - 强调文字颜色 4" xfId="40"/>
+    <x:cellStyle name="60% - 强调文字颜色 5" xfId="44"/>
+    <x:cellStyle name="60% - 强调文字颜色 6" xfId="48"/>
     <x:cellStyle name="百分比" xfId="3"/>
-    <x:cellStyle name="千位分隔[0]" xfId="4"/>
-    <x:cellStyle name="货币[0]" xfId="5"/>
-    <x:cellStyle name="超链接" xfId="6"/>
-    <x:cellStyle name="已访问的超链接" xfId="7"/>
-    <x:cellStyle name="注释" xfId="8"/>
-    <x:cellStyle name="警告文本" xfId="9"/>
     <x:cellStyle name="标题" xfId="10"/>
-    <x:cellStyle name="解释性文本" xfId="11"/>
     <x:cellStyle name="标题 1" xfId="12"/>
     <x:cellStyle name="标题 2" xfId="13"/>
     <x:cellStyle name="标题 3" xfId="14"/>
     <x:cellStyle name="标题 4" xfId="15"/>
-    <x:cellStyle name="输入" xfId="16"/>
-    <x:cellStyle name="输出" xfId="17"/>
+    <x:cellStyle name="差" xfId="23"/>
+    <x:cellStyle name="常规" xfId="0"/>
+    <x:cellStyle name="超链接" xfId="6"/>
+    <x:cellStyle name="好" xfId="22"/>
+    <x:cellStyle name="汇总" xfId="21"/>
+    <x:cellStyle name="货币" xfId="2"/>
+    <x:cellStyle name="货币[0]" xfId="5"/>
     <x:cellStyle name="计算" xfId="18"/>
     <x:cellStyle name="检查单元格" xfId="19"/>
+    <x:cellStyle name="解释性文本" xfId="11"/>
+    <x:cellStyle name="警告文本" xfId="9"/>
     <x:cellStyle name="链接单元格" xfId="20"/>
-    <x:cellStyle name="汇总" xfId="21"/>
-    <x:cellStyle name="好" xfId="22"/>
-    <x:cellStyle name="差" xfId="23"/>
+    <x:cellStyle name="千位分隔" xfId="1"/>
+    <x:cellStyle name="千位分隔[0]" xfId="4"/>
+    <x:cellStyle name="强调文字颜色 1" xfId="25"/>
+    <x:cellStyle name="强调文字颜色 2" xfId="29"/>
+    <x:cellStyle name="强调文字颜色 3" xfId="33"/>
+    <x:cellStyle name="强调文字颜色 4" xfId="37"/>
+    <x:cellStyle name="强调文字颜色 5" xfId="41"/>
+    <x:cellStyle name="强调文字颜色 6" xfId="45"/>
     <x:cellStyle name="适中" xfId="24"/>
-    <x:cellStyle name="强调文字颜色 1" xfId="25"/>
-    <x:cellStyle name="20% - 强调文字颜色 1" xfId="26"/>
-    <x:cellStyle name="40% - 强调文字颜色 1" xfId="27"/>
-    <x:cellStyle name="60% - 强调文字颜色 1" xfId="28"/>
-    <x:cellStyle name="强调文字颜色 2" xfId="29"/>
-    <x:cellStyle name="20% - 强调文字颜色 2" xfId="30"/>
-    <x:cellStyle name="40% - 强调文字颜色 2" xfId="31"/>
-    <x:cellStyle name="60% - 强调文字颜色 2" xfId="32"/>
-    <x:cellStyle name="强调文字颜色 3" xfId="33"/>
-    <x:cellStyle name="20% - 强调文字颜色 3" xfId="34"/>
-    <x:cellStyle name="40% - 强调文字颜色 3" xfId="35"/>
-    <x:cellStyle name="60% - 强调文字颜色 3" xfId="36"/>
-    <x:cellStyle name="强调文字颜色 4" xfId="37"/>
-    <x:cellStyle name="20% - 强调文字颜色 4" xfId="38"/>
-    <x:cellStyle name="40% - 强调文字颜色 4" xfId="39"/>
-    <x:cellStyle name="60% - 强调文字颜色 4" xfId="40"/>
-    <x:cellStyle name="强调文字颜色 5" xfId="41"/>
-    <x:cellStyle name="20% - 强调文字颜色 5" xfId="42"/>
-    <x:cellStyle name="40% - 强调文字颜色 5" xfId="43"/>
-    <x:cellStyle name="60% - 强调文字颜色 5" xfId="44"/>
-    <x:cellStyle name="强调文字颜色 6" xfId="45"/>
-    <x:cellStyle name="20% - 强调文字颜色 6" xfId="46"/>
-    <x:cellStyle name="40% - 强调文字颜色 6" xfId="47"/>
-    <x:cellStyle name="60% - 强调文字颜色 6" xfId="48"/>
+    <x:cellStyle name="输出" xfId="17"/>
+    <x:cellStyle name="输入" xfId="16"/>
+    <x:cellStyle name="样式 1" xfId="49"/>
+    <x:cellStyle name="已访问的超链接" xfId="7"/>
+    <x:cellStyle name="注释" xfId="8"/>
   </x:cellStyles>
-  <x:dxfs count="18">
+  <x:dxfs count="1">
     <x:dxf>
       <x:fill>
         <x:patternFill>
-          <x:bgColor theme="8" tint="0.6"/>
+          <x:bgColor theme="8" tint="0.59999"/>
         </x:patternFill>
       </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor theme="4" tint="0.79998"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor theme="4" tint="0.79998"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color theme="1"/>
-      </x:font>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color theme="1"/>
-      </x:font>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color theme="1"/>
-      </x:font>
-      <x:border>
-        <x:top style="double">
-          <x:color theme="4"/>
-        </x:top>
-      </x:border>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color theme="0"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor theme="4"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color theme="1"/>
-      </x:font>
-      <x:border>
-        <x:left style="thin">
-          <x:color theme="4"/>
-        </x:left>
-        <x:right style="thin">
-          <x:color theme="4"/>
-        </x:right>
-        <x:top style="thin">
-          <x:color theme="4"/>
-        </x:top>
-        <x:bottom style="thin">
-          <x:color theme="4"/>
-        </x:bottom>
-      </x:border>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor theme="4" tint="0.79998"/>
-        </x:patternFill>
-      </x:fill>
-      <x:border>
-        <x:bottom style="thin">
-          <x:color theme="4" tint="0.39998"/>
-        </x:bottom>
-      </x:border>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor theme="4" tint="0.79998"/>
-        </x:patternFill>
-      </x:fill>
-      <x:border>
-        <x:bottom style="thin">
-          <x:color theme="4" tint="0.39998"/>
-        </x:bottom>
-      </x:border>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color theme="1"/>
-      </x:font>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color theme="1"/>
-      </x:font>
-      <x:border>
-        <x:bottom style="thin">
-          <x:color theme="4" tint="0.39998"/>
-        </x:bottom>
-      </x:border>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color theme="1"/>
-      </x:font>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color theme="1"/>
-      </x:font>
-      <x:border>
-        <x:top style="thin">
-          <x:color theme="4"/>
-        </x:top>
-        <x:bottom style="thin">
-          <x:color theme="4"/>
-        </x:bottom>
-      </x:border>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor theme="4" tint="0.79998"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor theme="4" tint="0.79998"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color theme="1"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor theme="4" tint="0.79998"/>
-        </x:patternFill>
-      </x:fill>
-      <x:border>
-        <x:top style="thin">
-          <x:color theme="4" tint="0.39998"/>
-        </x:top>
-        <x:bottom style="thin">
-          <x:color theme="4" tint="0.39998"/>
-        </x:bottom>
-      </x:border>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color theme="1"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor theme="4" tint="0.79998"/>
-        </x:patternFill>
-      </x:fill>
-      <x:border>
-        <x:bottom style="thin">
-          <x:color theme="4" tint="0.39998"/>
-        </x:bottom>
-      </x:border>
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
@@ -3156,56 +3016,56 @@
   <x:sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <x:cols>
     <x:col min="2" max="2" width="14.625" customWidth="1"/>
-    <x:col min="3" max="3" width="19.25" style="2" customWidth="1"/>
+    <x:col min="3" max="3" width="26.25" style="2" customWidth="1"/>
     <x:col min="4" max="4" width="36" customWidth="1"/>
     <x:col min="5" max="5" width="42.625" customWidth="1"/>
     <x:col min="6" max="6" width="27.125" customWidth="1"/>
     <x:col min="7" max="7" width="36" customWidth="1"/>
     <x:col min="8" max="8" width="22.625" customWidth="1"/>
     <x:col min="9" max="9" width="31.5" customWidth="1"/>
-    <x:col min="10" max="10" width="8.375" customWidth="1"/>
-    <x:col min="11" max="11" width="8.625" customWidth="1"/>
-    <x:col min="12" max="12" width="8.125" customWidth="1"/>
+    <x:col min="10" max="10" width="20" customWidth="1"/>
+    <x:col min="11" max="11" width="15.875" customWidth="1"/>
+    <x:col min="12" max="12" width="13.625" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" s="1" customFormat="1" ht="27">
-      <x:c r="A1" s="3" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="3" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C1" s="4" t="s">
+    <x:row r="1" s="1" customFormat="1" ht="35.25">
+      <x:c r="A1" s="8" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="8" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C1" s="9" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="s">
+      <x:c r="D1" s="8" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="s">
+      <x:c r="E1" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="s">
+      <x:c r="F1" s="8" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G1" s="3" t="s">
+      <x:c r="G1" s="8" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="H1" s="3" t="s">
+      <x:c r="H1" s="8" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="I1" s="3" t="s">
+      <x:c r="I1" s="8" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="J1" s="3" t="s">
+      <x:c r="J1" s="8" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="K1" s="3" t="s">
+      <x:c r="K1" s="8" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="L1" s="3" t="s">
+      <x:c r="L1" s="8" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="M1" s="3" t="s">
+      <x:c r="M1" s="8" t="s">
         <x:v>12</x:v>
       </x:c>
     </x:row>
@@ -3213,28 +3073,28 @@
       <x:c r="A2">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="s">
+      <x:c r="B2" s="3" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C2" s="6">
+      <x:c r="C2" s="4">
         <x:v>41110</x:v>
       </x:c>
-      <x:c r="D2" s="7" t="s">
+      <x:c r="D2" s="5" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="E2" s="7" t="s">
+      <x:c r="E2" s="5" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F2" s="7" t="s">
+      <x:c r="F2" s="5" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="G2" s="7" t="s">
+      <x:c r="G2" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H2" s="7" t="s">
+      <x:c r="H2" s="5" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I2" s="7" t="s">
+      <x:c r="I2" s="5" t="s">
         <x:v>19</x:v>
       </x:c>
       <x:c r="J2">
@@ -3254,28 +3114,28 @@
       <x:c r="A3">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="s">
+      <x:c r="B3" s="3" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C3" s="6">
+      <x:c r="C3" s="4">
         <x:v>43469</x:v>
       </x:c>
-      <x:c r="D3" s="7" t="s">
+      <x:c r="D3" s="5" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="E3" s="7" t="s">
+      <x:c r="E3" s="5" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="F3" s="7" t="s">
+      <x:c r="F3" s="5" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="G3" s="7" t="s">
+      <x:c r="G3" s="5" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="H3" s="7" t="s">
+      <x:c r="H3" s="5" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="I3" s="7" t="s">
+      <x:c r="I3" s="5" t="s">
         <x:v>25</x:v>
       </x:c>
       <x:c r="J3">
@@ -3295,28 +3155,28 @@
       <x:c r="A4">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="s">
+      <x:c r="B4" s="3" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="C4" s="6">
+      <x:c r="C4" s="4">
         <x:v>45788</x:v>
       </x:c>
-      <x:c r="D4" s="7" t="s">
+      <x:c r="D4" s="5" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E4" s="7" t="s">
+      <x:c r="E4" s="5" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="F4" s="7" t="s">
+      <x:c r="F4" s="5" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="G4" s="7" t="s">
+      <x:c r="G4" s="5" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="H4" s="7" t="s">
+      <x:c r="H4" s="5" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="I4" s="7" t="s">
+      <x:c r="I4" s="5" t="s">
         <x:v>31</x:v>
       </x:c>
       <x:c r="J4">
@@ -3336,28 +3196,28 @@
       <x:c r="A5">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="s">
+      <x:c r="B5" s="3" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C5" s="6">
+      <x:c r="C5" s="4">
         <x:v>42189</x:v>
       </x:c>
-      <x:c r="D5" s="7" t="s">
+      <x:c r="D5" s="5" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="E5" s="7" t="s">
+      <x:c r="E5" s="5" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="F5" s="7" t="s">
+      <x:c r="F5" s="5" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="G5" s="7" t="s">
+      <x:c r="G5" s="5" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="H5" s="7" t="s">
+      <x:c r="H5" s="5" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="I5" s="7" t="s">
+      <x:c r="I5" s="5" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="J5">
@@ -3377,28 +3237,28 @@
       <x:c r="A6">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
+      <x:c r="B6" s="3" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C6" s="6">
+      <x:c r="C6" s="4">
         <x:v>43765</x:v>
       </x:c>
-      <x:c r="D6" s="7" t="s">
+      <x:c r="D6" s="5" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="E6" s="7" t="s">
+      <x:c r="E6" s="5" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="F6" s="7" t="s">
+      <x:c r="F6" s="5" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="G6" s="7" t="s">
+      <x:c r="G6" s="5" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="H6" s="7" t="s">
+      <x:c r="H6" s="5" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="I6" s="7" t="s">
+      <x:c r="I6" s="5" t="s">
         <x:v>45</x:v>
       </x:c>
       <x:c r="J6">
@@ -3418,28 +3278,28 @@
       <x:c r="A7">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="s">
+      <x:c r="B7" s="3" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="C7" s="6">
+      <x:c r="C7" s="4">
         <x:v>43780</x:v>
       </x:c>
-      <x:c r="D7" s="7" t="s">
+      <x:c r="D7" s="5" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="E7" s="7" t="s">
+      <x:c r="E7" s="5" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="F7" s="7" t="s">
+      <x:c r="F7" s="5" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="G7" s="7" t="s">
+      <x:c r="G7" s="5" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="H7" s="7" t="s">
+      <x:c r="H7" s="5" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="I7" s="7" t="s">
+      <x:c r="I7" s="5" t="s">
         <x:v>52</x:v>
       </x:c>
       <x:c r="J7">
@@ -3459,28 +3319,28 @@
       <x:c r="A8">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="s">
+      <x:c r="B8" s="3" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="C8" s="6">
+      <x:c r="C8" s="4">
         <x:v>43914</x:v>
       </x:c>
-      <x:c r="D8" s="7" t="s">
+      <x:c r="D8" s="5" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="E8" s="7" t="s">
+      <x:c r="E8" s="5" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="F8" s="7" t="s">
+      <x:c r="F8" s="5" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="G8" s="7" t="s">
+      <x:c r="G8" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="H8" s="7" t="s">
+      <x:c r="H8" s="5" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="I8" s="7" t="s">
+      <x:c r="I8" s="5" t="s">
         <x:v>59</x:v>
       </x:c>
       <x:c r="J8">
@@ -3500,28 +3360,28 @@
       <x:c r="A9">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="s">
+      <x:c r="B9" s="3" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="C9" s="6">
+      <x:c r="C9" s="4">
         <x:v>44036</x:v>
       </x:c>
-      <x:c r="D9" s="7" t="s">
+      <x:c r="D9" s="5" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="E9" s="7" t="s">
+      <x:c r="E9" s="5" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="F9" s="7" t="s">
+      <x:c r="F9" s="5" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="G9" s="7" t="s">
+      <x:c r="G9" s="5" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="H9" s="7" t="s">
+      <x:c r="H9" s="5" t="s">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="I9" s="7" t="s">
+      <x:c r="I9" s="5" t="s">
         <x:v>63</x:v>
       </x:c>
       <x:c r="J9">
@@ -3541,28 +3401,28 @@
       <x:c r="A10">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
+      <x:c r="B10" s="3" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="C10" s="6">
+      <x:c r="C10" s="4">
         <x:v>42369</x:v>
       </x:c>
-      <x:c r="D10" s="7" t="s">
+      <x:c r="D10" s="5" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="E10" s="7" t="s">
+      <x:c r="E10" s="5" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="F10" s="7" t="s">
+      <x:c r="F10" s="5" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="G10" s="7" t="s">
+      <x:c r="G10" s="5" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="H10" s="7" t="s">
+      <x:c r="H10" s="5" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="I10" s="7" t="s">
+      <x:c r="I10" s="5" t="s">
         <x:v>70</x:v>
       </x:c>
       <x:c r="J10">
@@ -3582,28 +3442,28 @@
       <x:c r="A11">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B11" s="5" t="s">
+      <x:c r="B11" s="3" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="C11" s="6">
+      <x:c r="C11" s="4">
         <x:v>43190</x:v>
       </x:c>
-      <x:c r="D11" s="7" t="s">
+      <x:c r="D11" s="5" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="E11" s="7" t="s">
+      <x:c r="E11" s="5" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="F11" s="7" t="s">
+      <x:c r="F11" s="5" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="G11" s="7" t="s">
+      <x:c r="G11" s="5" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="H11" s="7" t="s">
+      <x:c r="H11" s="5" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="I11" s="7" t="s">
+      <x:c r="I11" s="5" t="s">
         <x:v>77</x:v>
       </x:c>
       <x:c r="J11">
@@ -3623,28 +3483,28 @@
       <x:c r="A12">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
+      <x:c r="B12" s="3" t="s">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="C12" s="6">
+      <x:c r="C12" s="4">
         <x:v>41117</x:v>
       </x:c>
-      <x:c r="D12" s="7" t="s">
+      <x:c r="D12" s="5" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="E12" s="7" t="s">
+      <x:c r="E12" s="5" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="F12" s="7" t="s">
+      <x:c r="F12" s="5" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="G12" s="7" t="s">
+      <x:c r="G12" s="5" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="H12" s="7" t="s">
+      <x:c r="H12" s="5" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="I12" s="7" t="s">
+      <x:c r="I12" s="5" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="J12">
@@ -3664,28 +3524,28 @@
       <x:c r="A13">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="s">
+      <x:c r="B13" s="3" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="C13" s="6">
+      <x:c r="C13" s="4">
         <x:v>42098</x:v>
       </x:c>
-      <x:c r="D13" s="7" t="s">
+      <x:c r="D13" s="5" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="E13" s="7" t="s">
+      <x:c r="E13" s="5" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="F13" s="7" t="s">
+      <x:c r="F13" s="5" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="G13" s="7" t="s">
+      <x:c r="G13" s="5" t="s">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="H13" s="7" t="s">
+      <x:c r="H13" s="5" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="I13" s="7" t="s">
+      <x:c r="I13" s="5" t="s">
         <x:v>91</x:v>
       </x:c>
       <x:c r="J13">
@@ -3705,28 +3565,28 @@
       <x:c r="A14">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="s">
+      <x:c r="B14" s="3" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="C14" s="6">
+      <x:c r="C14" s="4">
         <x:v>43926</x:v>
       </x:c>
-      <x:c r="D14" s="7" t="s">
+      <x:c r="D14" s="5" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="E14" s="7" t="s">
+      <x:c r="E14" s="5" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="F14" s="7" t="s">
+      <x:c r="F14" s="5" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="G14" s="7" t="s">
+      <x:c r="G14" s="5" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="H14" s="7" t="s">
+      <x:c r="H14" s="5" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="I14" s="7" t="s">
+      <x:c r="I14" s="5" t="s">
         <x:v>97</x:v>
       </x:c>
       <x:c r="J14">
@@ -3746,28 +3606,28 @@
       <x:c r="A15">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="s">
+      <x:c r="B15" s="3" t="s">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="C15" s="6">
+      <x:c r="C15" s="4">
         <x:v>42770</x:v>
       </x:c>
-      <x:c r="D15" s="7" t="s">
+      <x:c r="D15" s="5" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="E15" s="7" t="s">
+      <x:c r="E15" s="5" t="s">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="F15" s="7" t="s">
+      <x:c r="F15" s="5" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="G15" s="7" t="s">
+      <x:c r="G15" s="5" t="s">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="H15" s="7" t="s">
+      <x:c r="H15" s="5" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="I15" s="7" t="s">
+      <x:c r="I15" s="5" t="s">
         <x:v>104</x:v>
       </x:c>
       <x:c r="J15">
@@ -3787,28 +3647,28 @@
       <x:c r="A16">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="s">
+      <x:c r="B16" s="3" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="C16" s="6">
+      <x:c r="C16" s="4">
         <x:v>41133</x:v>
       </x:c>
-      <x:c r="D16" s="7" t="s">
+      <x:c r="D16" s="5" t="s">
         <x:v>106</x:v>
       </x:c>
-      <x:c r="E16" s="7" t="s">
+      <x:c r="E16" s="5" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="F16" s="7" t="s">
+      <x:c r="F16" s="5" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="G16" s="7" t="s">
+      <x:c r="G16" s="5" t="s">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="H16" s="7" t="s">
+      <x:c r="H16" s="5" t="s">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="I16" s="7" t="s">
+      <x:c r="I16" s="5" t="s">
         <x:v>111</x:v>
       </x:c>
       <x:c r="J16">
@@ -3828,28 +3688,28 @@
       <x:c r="A17">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B17" s="5" t="s">
+      <x:c r="B17" s="3" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="C17" s="6">
+      <x:c r="C17" s="4">
         <x:v>41571</x:v>
       </x:c>
-      <x:c r="D17" s="7" t="s">
+      <x:c r="D17" s="5" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="E17" s="7" t="s">
+      <x:c r="E17" s="5" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="F17" s="7" t="s">
+      <x:c r="F17" s="5" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="G17" s="7" t="s">
+      <x:c r="G17" s="5" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="H17" s="7" t="s">
+      <x:c r="H17" s="5" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="I17" s="7" t="s">
+      <x:c r="I17" s="5" t="s">
         <x:v>118</x:v>
       </x:c>
       <x:c r="J17">
@@ -3869,28 +3729,28 @@
       <x:c r="A18">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="s">
+      <x:c r="B18" s="3" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="C18" s="6">
+      <x:c r="C18" s="4">
         <x:v>42644</x:v>
       </x:c>
-      <x:c r="D18" s="7" t="s">
+      <x:c r="D18" s="5" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="E18" s="7" t="s">
+      <x:c r="E18" s="5" t="s">
         <x:v>121</x:v>
       </x:c>
-      <x:c r="F18" s="7" t="s">
+      <x:c r="F18" s="5" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="G18" s="7" t="s">
+      <x:c r="G18" s="5" t="s">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="H18" s="7" t="s">
+      <x:c r="H18" s="5" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="I18" s="7" t="s">
+      <x:c r="I18" s="5" t="s">
         <x:v>125</x:v>
       </x:c>
       <x:c r="J18">
@@ -3910,28 +3770,28 @@
       <x:c r="A19">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B19" s="5" t="s">
+      <x:c r="B19" s="3" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="C19" s="6">
+      <x:c r="C19" s="4">
         <x:v>41284</x:v>
       </x:c>
-      <x:c r="D19" s="7" t="s">
+      <x:c r="D19" s="5" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="E19" s="7" t="s">
+      <x:c r="E19" s="5" t="s">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F19" s="7" t="s">
+      <x:c r="F19" s="5" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="G19" s="7" t="s">
+      <x:c r="G19" s="5" t="s">
         <x:v>130</x:v>
       </x:c>
-      <x:c r="H19" s="7" t="s">
+      <x:c r="H19" s="5" t="s">
         <x:v>131</x:v>
       </x:c>
-      <x:c r="I19" s="7" t="s">
+      <x:c r="I19" s="5" t="s">
         <x:v>132</x:v>
       </x:c>
       <x:c r="J19">
@@ -3951,28 +3811,28 @@
       <x:c r="A20">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B20" s="5" t="s">
+      <x:c r="B20" s="3" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="C20" s="6">
+      <x:c r="C20" s="4">
         <x:v>41424</x:v>
       </x:c>
-      <x:c r="D20" s="7" t="s">
+      <x:c r="D20" s="5" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="E20" s="7" t="s">
+      <x:c r="E20" s="5" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="F20" s="7" t="s">
+      <x:c r="F20" s="5" t="s">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="G20" s="7" t="s">
+      <x:c r="G20" s="5" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="H20" s="7" t="s">
+      <x:c r="H20" s="5" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="I20" s="7" t="s">
+      <x:c r="I20" s="5" t="s">
         <x:v>139</x:v>
       </x:c>
       <x:c r="J20">
@@ -3992,28 +3852,28 @@
       <x:c r="A21">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B21" s="5" t="s">
+      <x:c r="B21" s="3" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="C21" s="6">
+      <x:c r="C21" s="4">
         <x:v>45781</x:v>
       </x:c>
-      <x:c r="D21" s="7" t="s">
+      <x:c r="D21" s="5" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="E21" s="7" t="s">
+      <x:c r="E21" s="5" t="s">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="F21" s="7" t="s">
+      <x:c r="F21" s="5" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="G21" s="7" t="s">
+      <x:c r="G21" s="5" t="s">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="H21" s="7" t="s">
+      <x:c r="H21" s="5" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="I21" s="7" t="s">
+      <x:c r="I21" s="5" t="s">
         <x:v>146</x:v>
       </x:c>
       <x:c r="J21">
@@ -4033,28 +3893,28 @@
       <x:c r="A22">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B22" s="5" t="s">
+      <x:c r="B22" s="3" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="C22" s="6">
+      <x:c r="C22" s="4">
         <x:v>42218</x:v>
       </x:c>
-      <x:c r="D22" s="7" t="s">
+      <x:c r="D22" s="5" t="s">
         <x:v>148</x:v>
       </x:c>
-      <x:c r="E22" s="7" t="s">
+      <x:c r="E22" s="5" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="F22" s="7" t="s">
+      <x:c r="F22" s="5" t="s">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="G22" s="7" t="s">
+      <x:c r="G22" s="5" t="s">
         <x:v>151</x:v>
       </x:c>
-      <x:c r="H22" s="7" t="s">
+      <x:c r="H22" s="5" t="s">
         <x:v>152</x:v>
       </x:c>
-      <x:c r="I22" s="7" t="s">
+      <x:c r="I22" s="5" t="s">
         <x:v>153</x:v>
       </x:c>
       <x:c r="J22">
@@ -4074,28 +3934,28 @@
       <x:c r="A23">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B23" s="5" t="s">
+      <x:c r="B23" s="3" t="s">
         <x:v>154</x:v>
       </x:c>
-      <x:c r="C23" s="6">
+      <x:c r="C23" s="4">
         <x:v>42552</x:v>
       </x:c>
-      <x:c r="D23" s="7" t="s">
+      <x:c r="D23" s="5" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="E23" s="7" t="s">
+      <x:c r="E23" s="5" t="s">
         <x:v>156</x:v>
       </x:c>
-      <x:c r="F23" s="7" t="s">
+      <x:c r="F23" s="5" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="G23" s="7" t="s">
+      <x:c r="G23" s="5" t="s">
         <x:v>158</x:v>
       </x:c>
-      <x:c r="H23" s="7" t="s">
+      <x:c r="H23" s="5" t="s">
         <x:v>159</x:v>
       </x:c>
-      <x:c r="I23" s="7" t="s">
+      <x:c r="I23" s="5" t="s">
         <x:v>160</x:v>
       </x:c>
       <x:c r="J23">
@@ -4115,28 +3975,28 @@
       <x:c r="A24">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B24" s="5" t="s">
+      <x:c r="B24" s="3" t="s">
         <x:v>161</x:v>
       </x:c>
-      <x:c r="C24" s="6">
+      <x:c r="C24" s="4">
         <x:v>42979</x:v>
       </x:c>
-      <x:c r="D24" s="7" t="s">
+      <x:c r="D24" s="5" t="s">
         <x:v>162</x:v>
       </x:c>
-      <x:c r="E24" s="7" t="s">
+      <x:c r="E24" s="5" t="s">
         <x:v>163</x:v>
       </x:c>
-      <x:c r="F24" s="7" t="s">
+      <x:c r="F24" s="5" t="s">
         <x:v>162</x:v>
       </x:c>
-      <x:c r="G24" s="7" t="s">
+      <x:c r="G24" s="5" t="s">
         <x:v>164</x:v>
       </x:c>
-      <x:c r="H24" s="7" t="s">
+      <x:c r="H24" s="5" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="I24" s="7" t="s">
+      <x:c r="I24" s="5" t="s">
         <x:v>166</x:v>
       </x:c>
       <x:c r="J24">
@@ -4148,36 +4008,36 @@
       <x:c r="L24">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M24">
-        <x:v>1</x:v>
+      <x:c r="M24" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="18.75" hidden="1">
       <x:c r="A25">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B25" s="5" t="s">
+      <x:c r="B25" s="3" t="s">
         <x:v>167</x:v>
       </x:c>
-      <x:c r="C25" s="6">
+      <x:c r="C25" s="4">
         <x:v>41128</x:v>
       </x:c>
-      <x:c r="D25" s="7" t="s">
+      <x:c r="D25" s="5" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="E25" s="7" t="s">
+      <x:c r="E25" s="5" t="s">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="F25" s="7" t="s">
+      <x:c r="F25" s="5" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="G25" s="7" t="s">
+      <x:c r="G25" s="5" t="s">
         <x:v>171</x:v>
       </x:c>
-      <x:c r="H25" s="7" t="s">
+      <x:c r="H25" s="5" t="s">
         <x:v>172</x:v>
       </x:c>
-      <x:c r="I25" s="7" t="s">
+      <x:c r="I25" s="5" t="s">
         <x:v>173</x:v>
       </x:c>
       <x:c r="J25">
@@ -4197,28 +4057,28 @@
       <x:c r="A26">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B26" s="5" t="s">
+      <x:c r="B26" s="3" t="s">
         <x:v>174</x:v>
       </x:c>
-      <x:c r="C26" s="6">
+      <x:c r="C26" s="4">
         <x:v>41587</x:v>
       </x:c>
-      <x:c r="D26" s="7" t="s">
+      <x:c r="D26" s="5" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="E26" s="7" t="s">
+      <x:c r="E26" s="5" t="s">
         <x:v>176</x:v>
       </x:c>
-      <x:c r="F26" s="7" t="s">
+      <x:c r="F26" s="5" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="G26" s="7" t="s">
+      <x:c r="G26" s="5" t="s">
         <x:v>175</x:v>
       </x:c>
-      <x:c r="H26" s="7" t="s">
+      <x:c r="H26" s="5" t="s">
         <x:v>178</x:v>
       </x:c>
-      <x:c r="I26" s="7" t="s">
+      <x:c r="I26" s="5" t="s">
         <x:v>179</x:v>
       </x:c>
       <x:c r="J26">
@@ -4238,28 +4098,28 @@
       <x:c r="A27">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B27" s="5" t="s">
+      <x:c r="B27" s="3" t="s">
         <x:v>180</x:v>
       </x:c>
-      <x:c r="C27" s="6">
+      <x:c r="C27" s="4">
         <x:v>42529</x:v>
       </x:c>
-      <x:c r="D27" s="7" t="s">
+      <x:c r="D27" s="5" t="s">
         <x:v>181</x:v>
       </x:c>
-      <x:c r="E27" s="7" t="s">
+      <x:c r="E27" s="5" t="s">
         <x:v>182</x:v>
       </x:c>
-      <x:c r="F27" s="7" t="s">
+      <x:c r="F27" s="5" t="s">
         <x:v>183</x:v>
       </x:c>
-      <x:c r="G27" s="7" t="s">
+      <x:c r="G27" s="5" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="H27" s="7" t="s">
+      <x:c r="H27" s="5" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="I27" s="7" t="s">
+      <x:c r="I27" s="5" t="s">
         <x:v>186</x:v>
       </x:c>
       <x:c r="J27">
@@ -4279,28 +4139,28 @@
       <x:c r="A28">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B28" s="5" t="s">
+      <x:c r="B28" s="3" t="s">
         <x:v>187</x:v>
       </x:c>
-      <x:c r="C28" s="6">
+      <x:c r="C28" s="4">
         <x:v>42470</x:v>
       </x:c>
-      <x:c r="D28" s="7" t="s">
+      <x:c r="D28" s="5" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="E28" s="7" t="s">
+      <x:c r="E28" s="5" t="s">
         <x:v>188</x:v>
       </x:c>
-      <x:c r="F28" s="7" t="s">
+      <x:c r="F28" s="5" t="s">
         <x:v>189</x:v>
       </x:c>
-      <x:c r="G28" s="7" t="s">
+      <x:c r="G28" s="5" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="H28" s="7" t="s">
+      <x:c r="H28" s="5" t="s">
         <x:v>191</x:v>
       </x:c>
-      <x:c r="I28" s="7" t="s">
+      <x:c r="I28" s="5" t="s">
         <x:v>192</x:v>
       </x:c>
       <x:c r="J28">
@@ -4320,28 +4180,28 @@
       <x:c r="A29">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B29" s="5" t="s">
+      <x:c r="B29" s="3" t="s">
         <x:v>193</x:v>
       </x:c>
-      <x:c r="C29" s="6">
+      <x:c r="C29" s="4">
         <x:v>41766</x:v>
       </x:c>
-      <x:c r="D29" s="7" t="s">
+      <x:c r="D29" s="5" t="s">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="E29" s="7" t="s">
+      <x:c r="E29" s="5" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="F29" s="7" t="s">
+      <x:c r="F29" s="5" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="G29" s="7" t="s">
+      <x:c r="G29" s="5" t="s">
         <x:v>197</x:v>
       </x:c>
-      <x:c r="H29" s="7" t="s">
+      <x:c r="H29" s="5" t="s">
         <x:v>198</x:v>
       </x:c>
-      <x:c r="I29" s="7" t="s">
+      <x:c r="I29" s="5" t="s">
         <x:v>199</x:v>
       </x:c>
       <x:c r="J29">
@@ -4361,35 +4221,35 @@
       <x:c r="A30">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B30" s="5" t="s">
+      <x:c r="B30" s="3" t="s">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="C30" s="6">
+      <x:c r="C30" s="4">
         <x:v>41103</x:v>
       </x:c>
-      <x:c r="D30" s="7" t="s">
+      <x:c r="D30" s="5" t="s">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="E30" s="7" t="s">
+      <x:c r="E30" s="5" t="s">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="F30" s="7" t="s">
+      <x:c r="F30" s="5" t="s">
         <x:v>202</x:v>
       </x:c>
-      <x:c r="G30" s="7" t="s">
+      <x:c r="G30" s="5" t="s">
         <x:v>203</x:v>
       </x:c>
-      <x:c r="H30" s="7" t="s">
+      <x:c r="H30" s="5" t="s">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="I30" s="7" t="s">
+      <x:c r="I30" s="5" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="J30">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K30">
-        <x:v>0</x:v>
+      <x:c r="K30" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L30">
         <x:v>0</x:v>
@@ -4402,28 +4262,28 @@
       <x:c r="A31">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B31" s="5" t="s">
+      <x:c r="B31" s="3" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="C31" s="6">
+      <x:c r="C31" s="4">
         <x:v>41433</x:v>
       </x:c>
-      <x:c r="D31" s="7" t="s">
+      <x:c r="D31" s="5" t="s">
         <x:v>207</x:v>
       </x:c>
-      <x:c r="E31" s="7" t="s">
+      <x:c r="E31" s="5" t="s">
         <x:v>208</x:v>
       </x:c>
-      <x:c r="F31" s="7" t="s">
+      <x:c r="F31" s="5" t="s">
         <x:v>209</x:v>
       </x:c>
-      <x:c r="G31" s="7" t="s">
+      <x:c r="G31" s="5" t="s">
         <x:v>210</x:v>
       </x:c>
-      <x:c r="H31" s="7" t="s">
+      <x:c r="H31" s="5" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="I31" s="7" t="s">
+      <x:c r="I31" s="5" t="s">
         <x:v>212</x:v>
       </x:c>
       <x:c r="J31">
@@ -4443,28 +4303,28 @@
       <x:c r="A32">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B32" s="5" t="s">
+      <x:c r="B32" s="3" t="s">
         <x:v>213</x:v>
       </x:c>
-      <x:c r="C32" s="6">
+      <x:c r="C32" s="4">
         <x:v>41107</x:v>
       </x:c>
-      <x:c r="D32" s="7" t="s">
+      <x:c r="D32" s="5" t="s">
         <x:v>214</x:v>
       </x:c>
-      <x:c r="E32" s="7" t="s">
+      <x:c r="E32" s="5" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="F32" s="7" t="s">
+      <x:c r="F32" s="5" t="s">
         <x:v>216</x:v>
       </x:c>
-      <x:c r="G32" s="7" t="s">
+      <x:c r="G32" s="5" t="s">
         <x:v>217</x:v>
       </x:c>
-      <x:c r="H32" s="7" t="s">
+      <x:c r="H32" s="5" t="s">
         <x:v>218</x:v>
       </x:c>
-      <x:c r="I32" s="7" t="s">
+      <x:c r="I32" s="5" t="s">
         <x:v>219</x:v>
       </x:c>
       <x:c r="J32">
@@ -4484,28 +4344,28 @@
       <x:c r="A33">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B33" s="5" t="s">
+      <x:c r="B33" s="3" t="s">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="C33" s="6">
+      <x:c r="C33" s="4">
         <x:v>42119</x:v>
       </x:c>
-      <x:c r="D33" s="7" t="s">
+      <x:c r="D33" s="5" t="s">
         <x:v>221</x:v>
       </x:c>
-      <x:c r="E33" s="7" t="s">
+      <x:c r="E33" s="5" t="s">
         <x:v>222</x:v>
       </x:c>
-      <x:c r="F33" s="7" t="s">
+      <x:c r="F33" s="5" t="s">
         <x:v>223</x:v>
       </x:c>
-      <x:c r="G33" s="7" t="s">
+      <x:c r="G33" s="5" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="H33" s="7" t="s">
+      <x:c r="H33" s="5" t="s">
         <x:v>225</x:v>
       </x:c>
-      <x:c r="I33" s="7" t="s">
+      <x:c r="I33" s="5" t="s">
         <x:v>226</x:v>
       </x:c>
       <x:c r="J33">
@@ -4525,28 +4385,28 @@
       <x:c r="A34">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B34" s="5" t="s">
+      <x:c r="B34" s="3" t="s">
         <x:v>227</x:v>
       </x:c>
-      <x:c r="C34" s="6">
+      <x:c r="C34" s="4">
         <x:v>41889</x:v>
       </x:c>
-      <x:c r="D34" s="7" t="s">
+      <x:c r="D34" s="5" t="s">
         <x:v>228</x:v>
       </x:c>
-      <x:c r="E34" s="7" t="s">
+      <x:c r="E34" s="5" t="s">
         <x:v>229</x:v>
       </x:c>
-      <x:c r="F34" s="7" t="s">
+      <x:c r="F34" s="5" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="G34" s="7" t="s">
+      <x:c r="G34" s="5" t="s">
         <x:v>231</x:v>
       </x:c>
-      <x:c r="H34" s="7" t="s">
+      <x:c r="H34" s="5" t="s">
         <x:v>232</x:v>
       </x:c>
-      <x:c r="I34" s="7" t="s">
+      <x:c r="I34" s="5" t="s">
         <x:v>233</x:v>
       </x:c>
       <x:c r="J34">
@@ -4566,28 +4426,28 @@
       <x:c r="A35">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="B35" s="5" t="s">
+      <x:c r="B35" s="3" t="s">
         <x:v>234</x:v>
       </x:c>
-      <x:c r="C35" s="6">
+      <x:c r="C35" s="4">
         <x:v>41236</x:v>
       </x:c>
-      <x:c r="D35" s="7" t="s">
+      <x:c r="D35" s="5" t="s">
         <x:v>235</x:v>
       </x:c>
-      <x:c r="E35" s="7" t="s">
+      <x:c r="E35" s="5" t="s">
         <x:v>235</x:v>
       </x:c>
-      <x:c r="F35" s="7" t="s">
+      <x:c r="F35" s="5" t="s">
         <x:v>236</x:v>
       </x:c>
-      <x:c r="G35" s="7" t="s">
+      <x:c r="G35" s="5" t="s">
         <x:v>237</x:v>
       </x:c>
-      <x:c r="H35" s="7" t="s">
+      <x:c r="H35" s="5" t="s">
         <x:v>238</x:v>
       </x:c>
-      <x:c r="I35" s="7" t="s">
+      <x:c r="I35" s="5" t="s">
         <x:v>239</x:v>
       </x:c>
       <x:c r="J35">
@@ -4607,28 +4467,28 @@
       <x:c r="A36">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B36" s="5" t="s">
+      <x:c r="B36" s="3" t="s">
         <x:v>240</x:v>
       </x:c>
-      <x:c r="C36" s="6">
+      <x:c r="C36" s="4">
         <x:v>41635</x:v>
       </x:c>
-      <x:c r="D36" s="7" t="s">
+      <x:c r="D36" s="5" t="s">
         <x:v>241</x:v>
       </x:c>
-      <x:c r="E36" s="7" t="s">
+      <x:c r="E36" s="5" t="s">
         <x:v>242</x:v>
       </x:c>
-      <x:c r="F36" s="7" t="s">
+      <x:c r="F36" s="5" t="s">
         <x:v>243</x:v>
       </x:c>
-      <x:c r="G36" s="7" t="s">
+      <x:c r="G36" s="5" t="s">
         <x:v>244</x:v>
       </x:c>
-      <x:c r="H36" s="7" t="s">
+      <x:c r="H36" s="5" t="s">
         <x:v>245</x:v>
       </x:c>
-      <x:c r="I36" s="7" t="s">
+      <x:c r="I36" s="5" t="s">
         <x:v>246</x:v>
       </x:c>
       <x:c r="J36">
@@ -4640,36 +4500,36 @@
       <x:c r="L36">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M36">
-        <x:v>0</x:v>
+      <x:c r="M36" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="18.75">
       <x:c r="A37">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B37" s="5" t="s">
+      <x:c r="B37" s="3" t="s">
         <x:v>247</x:v>
       </x:c>
-      <x:c r="C37" s="6">
+      <x:c r="C37" s="4">
         <x:v>41867</x:v>
       </x:c>
-      <x:c r="D37" s="7" t="s">
+      <x:c r="D37" s="5" t="s">
         <x:v>248</x:v>
       </x:c>
-      <x:c r="E37" s="7" t="s">
+      <x:c r="E37" s="5" t="s">
         <x:v>249</x:v>
       </x:c>
-      <x:c r="F37" s="7" t="s">
+      <x:c r="F37" s="5" t="s">
         <x:v>250</x:v>
       </x:c>
-      <x:c r="G37" s="7" t="s">
+      <x:c r="G37" s="5" t="s">
         <x:v>251</x:v>
       </x:c>
-      <x:c r="H37" s="7" t="s">
+      <x:c r="H37" s="5" t="s">
         <x:v>252</x:v>
       </x:c>
-      <x:c r="I37" s="7" t="s">
+      <x:c r="I37" s="5" t="s">
         <x:v>253</x:v>
       </x:c>
       <x:c r="J37">
@@ -4689,28 +4549,28 @@
       <x:c r="A38">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B38" s="5" t="s">
+      <x:c r="B38" s="3" t="s">
         <x:v>254</x:v>
       </x:c>
-      <x:c r="C38" s="6">
+      <x:c r="C38" s="4">
         <x:v>41109</x:v>
       </x:c>
-      <x:c r="D38" s="7" t="s">
+      <x:c r="D38" s="5" t="s">
         <x:v>255</x:v>
       </x:c>
-      <x:c r="E38" s="7" t="s">
+      <x:c r="E38" s="5" t="s">
         <x:v>256</x:v>
       </x:c>
-      <x:c r="F38" s="7" t="s">
+      <x:c r="F38" s="5" t="s">
         <x:v>257</x:v>
       </x:c>
-      <x:c r="G38" s="7" t="s">
+      <x:c r="G38" s="5" t="s">
         <x:v>258</x:v>
       </x:c>
-      <x:c r="H38" s="7" t="s">
+      <x:c r="H38" s="5" t="s">
         <x:v>259</x:v>
       </x:c>
-      <x:c r="I38" s="7" t="s">
+      <x:c r="I38" s="5" t="s">
         <x:v>260</x:v>
       </x:c>
       <x:c r="J38">
@@ -4730,28 +4590,28 @@
       <x:c r="A39">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="B39" s="5" t="s">
+      <x:c r="B39" s="3" t="s">
         <x:v>261</x:v>
       </x:c>
-      <x:c r="C39" s="6">
+      <x:c r="C39" s="4">
         <x:v>42433</x:v>
       </x:c>
-      <x:c r="D39" s="7" t="s">
+      <x:c r="D39" s="5" t="s">
         <x:v>262</x:v>
       </x:c>
-      <x:c r="E39" s="7" t="s">
+      <x:c r="E39" s="5" t="s">
         <x:v>263</x:v>
       </x:c>
-      <x:c r="F39" s="7" t="s">
+      <x:c r="F39" s="5" t="s">
         <x:v>264</x:v>
       </x:c>
-      <x:c r="G39" s="7" t="s">
+      <x:c r="G39" s="5" t="s">
         <x:v>265</x:v>
       </x:c>
-      <x:c r="H39" s="7" t="s">
+      <x:c r="H39" s="5" t="s">
         <x:v>266</x:v>
       </x:c>
-      <x:c r="I39" s="7" t="s">
+      <x:c r="I39" s="5" t="s">
         <x:v>267</x:v>
       </x:c>
       <x:c r="J39">
@@ -4771,28 +4631,28 @@
       <x:c r="A40">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B40" s="5" t="s">
+      <x:c r="B40" s="3" t="s">
         <x:v>268</x:v>
       </x:c>
-      <x:c r="C40" s="6">
+      <x:c r="C40" s="4">
         <x:v>41306</x:v>
       </x:c>
-      <x:c r="D40" s="7" t="s">
+      <x:c r="D40" s="5" t="s">
         <x:v>269</x:v>
       </x:c>
-      <x:c r="E40" s="7" t="s">
+      <x:c r="E40" s="5" t="s">
         <x:v>270</x:v>
       </x:c>
-      <x:c r="F40" s="7" t="s">
+      <x:c r="F40" s="5" t="s">
         <x:v>271</x:v>
       </x:c>
-      <x:c r="G40" s="7" t="s">
+      <x:c r="G40" s="5" t="s">
         <x:v>272</x:v>
       </x:c>
-      <x:c r="H40" s="7" t="s">
+      <x:c r="H40" s="5" t="s">
         <x:v>273</x:v>
       </x:c>
-      <x:c r="I40" s="7" t="s">
+      <x:c r="I40" s="5" t="s">
         <x:v>274</x:v>
       </x:c>
       <x:c r="J40">
@@ -4804,36 +4664,36 @@
       <x:c r="L40">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M40">
-        <x:v>0</x:v>
+      <x:c r="M40" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="18.75">
       <x:c r="A41">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="B41" s="5" t="s">
+      <x:c r="B41" s="3" t="s">
         <x:v>275</x:v>
       </x:c>
-      <x:c r="C41" s="6">
+      <x:c r="C41" s="4">
         <x:v>42404</x:v>
       </x:c>
-      <x:c r="D41" s="7" t="s">
+      <x:c r="D41" s="5" t="s">
         <x:v>276</x:v>
       </x:c>
-      <x:c r="E41" s="7" t="s">
+      <x:c r="E41" s="5" t="s">
         <x:v>277</x:v>
       </x:c>
-      <x:c r="F41" s="7" t="s">
+      <x:c r="F41" s="5" t="s">
         <x:v>278</x:v>
       </x:c>
-      <x:c r="G41" s="7" t="s">
+      <x:c r="G41" s="5" t="s">
         <x:v>279</x:v>
       </x:c>
-      <x:c r="H41" s="7" t="s">
+      <x:c r="H41" s="5" t="s">
         <x:v>280</x:v>
       </x:c>
-      <x:c r="I41" s="7" t="s">
+      <x:c r="I41" s="5" t="s">
         <x:v>281</x:v>
       </x:c>
       <x:c r="J41">
@@ -4853,28 +4713,28 @@
       <x:c r="A42">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B42" s="5" t="s">
+      <x:c r="B42" s="3" t="s">
         <x:v>282</x:v>
       </x:c>
-      <x:c r="C42" s="6">
+      <x:c r="C42" s="4">
         <x:v>42778</x:v>
       </x:c>
-      <x:c r="D42" s="7" t="s">
+      <x:c r="D42" s="5" t="s">
         <x:v>283</x:v>
       </x:c>
-      <x:c r="E42" s="7" t="s">
+      <x:c r="E42" s="5" t="s">
         <x:v>284</x:v>
       </x:c>
-      <x:c r="F42" s="7" t="s">
+      <x:c r="F42" s="5" t="s">
         <x:v>285</x:v>
       </x:c>
-      <x:c r="G42" s="7" t="s">
+      <x:c r="G42" s="5" t="s">
         <x:v>283</x:v>
       </x:c>
-      <x:c r="H42" s="7" t="s">
+      <x:c r="H42" s="5" t="s">
         <x:v>286</x:v>
       </x:c>
-      <x:c r="I42" s="7" t="s">
+      <x:c r="I42" s="5" t="s">
         <x:v>287</x:v>
       </x:c>
       <x:c r="J42">
@@ -4894,28 +4754,28 @@
       <x:c r="A43">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B43" s="5" t="s">
+      <x:c r="B43" s="3" t="s">
         <x:v>288</x:v>
       </x:c>
-      <x:c r="C43" s="6">
+      <x:c r="C43" s="4">
         <x:v>42295</x:v>
       </x:c>
-      <x:c r="D43" s="7" t="s">
+      <x:c r="D43" s="5" t="s">
         <x:v>289</x:v>
       </x:c>
-      <x:c r="E43" s="7" t="s">
+      <x:c r="E43" s="5" t="s">
         <x:v>290</x:v>
       </x:c>
-      <x:c r="F43" s="7" t="s">
+      <x:c r="F43" s="5" t="s">
         <x:v>291</x:v>
       </x:c>
-      <x:c r="G43" s="7" t="s">
+      <x:c r="G43" s="5" t="s">
         <x:v>292</x:v>
       </x:c>
-      <x:c r="H43" s="7" t="s">
+      <x:c r="H43" s="5" t="s">
         <x:v>293</x:v>
       </x:c>
-      <x:c r="I43" s="7" t="s">
+      <x:c r="I43" s="5" t="s">
         <x:v>294</x:v>
       </x:c>
       <x:c r="J43">
@@ -4935,28 +4795,28 @@
       <x:c r="A44">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B44" s="5" t="s">
+      <x:c r="B44" s="3" t="s">
         <x:v>295</x:v>
       </x:c>
-      <x:c r="C44" s="6">
+      <x:c r="C44" s="4">
         <x:v>42826</x:v>
       </x:c>
-      <x:c r="D44" s="7" t="s">
+      <x:c r="D44" s="5" t="s">
         <x:v>296</x:v>
       </x:c>
-      <x:c r="E44" s="7" t="s">
+      <x:c r="E44" s="5" t="s">
         <x:v>297</x:v>
       </x:c>
-      <x:c r="F44" s="7" t="s">
+      <x:c r="F44" s="5" t="s">
         <x:v>298</x:v>
       </x:c>
-      <x:c r="G44" s="7" t="s">
+      <x:c r="G44" s="5" t="s">
         <x:v>299</x:v>
       </x:c>
-      <x:c r="H44" s="7" t="s">
+      <x:c r="H44" s="5" t="s">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="I44" s="7" t="s">
+      <x:c r="I44" s="5" t="s">
         <x:v>301</x:v>
       </x:c>
       <x:c r="J44">
@@ -4976,28 +4836,28 @@
       <x:c r="A45">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="B45" s="5" t="s">
+      <x:c r="B45" s="3" t="s">
         <x:v>302</x:v>
       </x:c>
-      <x:c r="C45" s="6">
+      <x:c r="C45" s="4">
         <x:v>41224</x:v>
       </x:c>
-      <x:c r="D45" s="7" t="s">
+      <x:c r="D45" s="5" t="s">
         <x:v>303</x:v>
       </x:c>
-      <x:c r="E45" s="7" t="s">
+      <x:c r="E45" s="5" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="F45" s="7" t="s">
+      <x:c r="F45" s="5" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="G45" s="7" t="s">
+      <x:c r="G45" s="5" t="s">
         <x:v>304</x:v>
       </x:c>
-      <x:c r="H45" s="7" t="s">
+      <x:c r="H45" s="5" t="s">
         <x:v>305</x:v>
       </x:c>
-      <x:c r="I45" s="7" t="s">
+      <x:c r="I45" s="5" t="s">
         <x:v>306</x:v>
       </x:c>
       <x:c r="J45">
@@ -5017,28 +4877,28 @@
       <x:c r="A46">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B46" s="5" t="s">
+      <x:c r="B46" s="3" t="s">
         <x:v>307</x:v>
       </x:c>
-      <x:c r="C46" s="6">
+      <x:c r="C46" s="4">
         <x:v>42819</x:v>
       </x:c>
-      <x:c r="D46" s="7" t="s">
+      <x:c r="D46" s="5" t="s">
         <x:v>308</x:v>
       </x:c>
-      <x:c r="E46" s="7" t="s">
+      <x:c r="E46" s="5" t="s">
         <x:v>196</x:v>
       </x:c>
-      <x:c r="F46" s="7" t="s">
+      <x:c r="F46" s="5" t="s">
         <x:v>309</x:v>
       </x:c>
-      <x:c r="G46" s="7" t="s">
+      <x:c r="G46" s="5" t="s">
         <x:v>310</x:v>
       </x:c>
-      <x:c r="H46" s="7" t="s">
+      <x:c r="H46" s="5" t="s">
         <x:v>311</x:v>
       </x:c>
-      <x:c r="I46" s="7" t="s">
+      <x:c r="I46" s="5" t="s">
         <x:v>265</x:v>
       </x:c>
       <x:c r="J46">
@@ -5058,28 +4918,28 @@
       <x:c r="A47">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="B47" s="5" t="s">
+      <x:c r="B47" s="3" t="s">
         <x:v>312</x:v>
       </x:c>
-      <x:c r="C47" s="6">
+      <x:c r="C47" s="4">
         <x:v>41066</x:v>
       </x:c>
-      <x:c r="D47" s="7" t="s">
+      <x:c r="D47" s="5" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="E47" s="7" t="s">
+      <x:c r="E47" s="5" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="F47" s="7" t="s">
+      <x:c r="F47" s="5" t="s">
         <x:v>314</x:v>
       </x:c>
-      <x:c r="G47" s="7" t="s">
+      <x:c r="G47" s="5" t="s">
         <x:v>315</x:v>
       </x:c>
-      <x:c r="H47" s="7" t="s">
+      <x:c r="H47" s="5" t="s">
         <x:v>316</x:v>
       </x:c>
-      <x:c r="I47" s="7" t="s">
+      <x:c r="I47" s="5" t="s">
         <x:v>317</x:v>
       </x:c>
       <x:c r="J47">
@@ -5099,28 +4959,28 @@
       <x:c r="A48">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B48" s="5" t="s">
+      <x:c r="B48" s="3" t="s">
         <x:v>318</x:v>
       </x:c>
-      <x:c r="C48" s="6">
+      <x:c r="C48" s="4">
         <x:v>41108</x:v>
       </x:c>
-      <x:c r="D48" s="7" t="s">
+      <x:c r="D48" s="5" t="s">
         <x:v>319</x:v>
       </x:c>
-      <x:c r="E48" s="7" t="s">
+      <x:c r="E48" s="5" t="s">
         <x:v>320</x:v>
       </x:c>
-      <x:c r="F48" s="7" t="s">
+      <x:c r="F48" s="5" t="s">
         <x:v>321</x:v>
       </x:c>
-      <x:c r="G48" s="7" t="s">
+      <x:c r="G48" s="5" t="s">
         <x:v>322</x:v>
       </x:c>
-      <x:c r="H48" s="7" t="s">
+      <x:c r="H48" s="5" t="s">
         <x:v>323</x:v>
       </x:c>
-      <x:c r="I48" s="7" t="s">
+      <x:c r="I48" s="5" t="s">
         <x:v>324</x:v>
       </x:c>
       <x:c r="J48">
@@ -5140,28 +5000,28 @@
       <x:c r="A49">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="B49" s="5" t="s">
+      <x:c r="B49" s="3" t="s">
         <x:v>325</x:v>
       </x:c>
-      <x:c r="C49" s="9" t="n">
+      <x:c r="C49" s="7">
         <x:v>41310</x:v>
       </x:c>
-      <x:c r="D49" s="7" t="s">
+      <x:c r="D49" s="5" t="s">
         <x:v>326</x:v>
       </x:c>
-      <x:c r="E49" s="7" t="s">
+      <x:c r="E49" s="5" t="s">
         <x:v>326</x:v>
       </x:c>
-      <x:c r="F49" s="7" t="s">
+      <x:c r="F49" s="5" t="s">
         <x:v>327</x:v>
       </x:c>
-      <x:c r="G49" s="7" t="s">
+      <x:c r="G49" s="5" t="s">
         <x:v>328</x:v>
       </x:c>
-      <x:c r="H49" s="7" t="s">
+      <x:c r="H49" s="5" t="s">
         <x:v>329</x:v>
       </x:c>
-      <x:c r="I49" s="7" t="s">
+      <x:c r="I49" s="5" t="s">
         <x:v>330</x:v>
       </x:c>
       <x:c r="J49">
@@ -5181,28 +5041,28 @@
       <x:c r="A50">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="B50" s="5" t="s">
+      <x:c r="B50" s="3" t="s">
         <x:v>331</x:v>
       </x:c>
-      <x:c r="C50" s="6">
+      <x:c r="C50" s="4">
         <x:v>42581</x:v>
       </x:c>
-      <x:c r="D50" s="7" t="s">
+      <x:c r="D50" s="5" t="s">
         <x:v>332</x:v>
       </x:c>
-      <x:c r="E50" s="7" t="s">
+      <x:c r="E50" s="5" t="s">
         <x:v>333</x:v>
       </x:c>
-      <x:c r="F50" s="7" t="s">
+      <x:c r="F50" s="5" t="s">
         <x:v>334</x:v>
       </x:c>
-      <x:c r="G50" s="7" t="s">
+      <x:c r="G50" s="5" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="H50" s="7" t="s">
+      <x:c r="H50" s="5" t="s">
         <x:v>335</x:v>
       </x:c>
-      <x:c r="I50" s="7" t="s">
+      <x:c r="I50" s="5" t="s">
         <x:v>336</x:v>
       </x:c>
       <x:c r="J50">
@@ -5222,28 +5082,28 @@
       <x:c r="A51">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="B51" s="5" t="s">
+      <x:c r="B51" s="3" t="s">
         <x:v>337</x:v>
       </x:c>
-      <x:c r="C51" s="6">
+      <x:c r="C51" s="4">
         <x:v>45052</x:v>
       </x:c>
-      <x:c r="D51" s="7" t="s">
+      <x:c r="D51" s="5" t="s">
         <x:v>338</x:v>
       </x:c>
-      <x:c r="E51" s="7" t="s">
+      <x:c r="E51" s="5" t="s">
         <x:v>339</x:v>
       </x:c>
-      <x:c r="F51" s="7" t="s">
+      <x:c r="F51" s="5" t="s">
         <x:v>340</x:v>
       </x:c>
-      <x:c r="G51" s="7" t="s">
+      <x:c r="G51" s="5" t="s">
         <x:v>341</x:v>
       </x:c>
-      <x:c r="H51" s="7" t="s">
+      <x:c r="H51" s="5" t="s">
         <x:v>342</x:v>
       </x:c>
-      <x:c r="I51" s="7" t="s">
+      <x:c r="I51" s="5" t="s">
         <x:v>343</x:v>
       </x:c>
       <x:c r="J51">
@@ -5255,36 +5115,36 @@
       <x:c r="L51">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M51">
-        <x:v>0</x:v>
+      <x:c r="M51" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="18.75" hidden="1">
       <x:c r="A52">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B52" s="5" t="s">
+      <x:c r="B52" s="3" t="s">
         <x:v>344</x:v>
       </x:c>
-      <x:c r="C52" s="6">
+      <x:c r="C52" s="4">
         <x:v>42300</x:v>
       </x:c>
-      <x:c r="D52" s="7" t="s">
+      <x:c r="D52" s="5" t="s">
         <x:v>345</x:v>
       </x:c>
-      <x:c r="E52" s="7" t="s">
+      <x:c r="E52" s="5" t="s">
         <x:v>346</x:v>
       </x:c>
-      <x:c r="F52" s="7" t="s">
+      <x:c r="F52" s="5" t="s">
         <x:v>345</x:v>
       </x:c>
-      <x:c r="G52" s="7" t="s">
+      <x:c r="G52" s="5" t="s">
         <x:v>347</x:v>
       </x:c>
-      <x:c r="H52" s="7" t="s">
+      <x:c r="H52" s="5" t="s">
         <x:v>348</x:v>
       </x:c>
-      <x:c r="I52" s="7" t="s">
+      <x:c r="I52" s="5" t="s">
         <x:v>349</x:v>
       </x:c>
       <x:c r="J52">
@@ -5304,28 +5164,28 @@
       <x:c r="A53">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="B53" s="5" t="s">
+      <x:c r="B53" s="3" t="s">
         <x:v>350</x:v>
       </x:c>
-      <x:c r="C53" s="6">
+      <x:c r="C53" s="4">
         <x:v>43875</x:v>
       </x:c>
-      <x:c r="D53" s="7" t="s">
+      <x:c r="D53" s="5" t="s">
         <x:v>351</x:v>
       </x:c>
-      <x:c r="E53" s="7" t="s">
+      <x:c r="E53" s="5" t="s">
         <x:v>352</x:v>
       </x:c>
-      <x:c r="F53" s="7" t="s">
+      <x:c r="F53" s="5" t="s">
         <x:v>353</x:v>
       </x:c>
-      <x:c r="G53" s="7" t="s">
+      <x:c r="G53" s="5" t="s">
         <x:v>354</x:v>
       </x:c>
-      <x:c r="H53" s="7" t="s">
+      <x:c r="H53" s="5" t="s">
         <x:v>355</x:v>
       </x:c>
-      <x:c r="I53" s="7" t="s">
+      <x:c r="I53" s="5" t="s">
         <x:v>356</x:v>
       </x:c>
       <x:c r="J53">
@@ -5345,28 +5205,28 @@
       <x:c r="A54">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="B54" s="5" t="s">
+      <x:c r="B54" s="3" t="s">
         <x:v>357</x:v>
       </x:c>
-      <x:c r="C54" s="6">
+      <x:c r="C54" s="4">
         <x:v>41408</x:v>
       </x:c>
-      <x:c r="D54" s="7" t="s">
+      <x:c r="D54" s="5" t="s">
         <x:v>358</x:v>
       </x:c>
-      <x:c r="E54" s="7" t="s">
+      <x:c r="E54" s="5" t="s">
         <x:v>359</x:v>
       </x:c>
-      <x:c r="F54" s="8">
+      <x:c r="F54" s="6">
         <x:v>7305</x:v>
       </x:c>
-      <x:c r="G54" s="7" t="s">
+      <x:c r="G54" s="5" t="s">
         <x:v>360</x:v>
       </x:c>
-      <x:c r="H54" s="7" t="s">
+      <x:c r="H54" s="5" t="s">
         <x:v>361</x:v>
       </x:c>
-      <x:c r="I54" s="7" t="s">
+      <x:c r="I54" s="5" t="s">
         <x:v>362</x:v>
       </x:c>
       <x:c r="J54">
@@ -5386,28 +5246,28 @@
       <x:c r="A55">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="B55" s="5" t="s">
+      <x:c r="B55" s="3" t="s">
         <x:v>363</x:v>
       </x:c>
-      <x:c r="C55" s="6">
+      <x:c r="C55" s="4">
         <x:v>43027</x:v>
       </x:c>
-      <x:c r="D55" s="7" t="s">
+      <x:c r="D55" s="5" t="s">
         <x:v>364</x:v>
       </x:c>
-      <x:c r="E55" s="7" t="s">
+      <x:c r="E55" s="5" t="s">
         <x:v>365</x:v>
       </x:c>
-      <x:c r="F55" s="7" t="s">
+      <x:c r="F55" s="5" t="s">
         <x:v>366</x:v>
       </x:c>
-      <x:c r="G55" s="7" t="s">
+      <x:c r="G55" s="5" t="s">
         <x:v>367</x:v>
       </x:c>
-      <x:c r="H55" s="7" t="s">
+      <x:c r="H55" s="5" t="s">
         <x:v>368</x:v>
       </x:c>
-      <x:c r="I55" s="7" t="s">
+      <x:c r="I55" s="5" t="s">
         <x:v>369</x:v>
       </x:c>
       <x:c r="J55">
@@ -5427,28 +5287,28 @@
       <x:c r="A56">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="B56" s="5" t="s">
+      <x:c r="B56" s="3" t="s">
         <x:v>370</x:v>
       </x:c>
-      <x:c r="C56" s="6">
+      <x:c r="C56" s="4">
         <x:v>42238</x:v>
       </x:c>
-      <x:c r="D56" s="7" t="s">
+      <x:c r="D56" s="5" t="s">
         <x:v>371</x:v>
       </x:c>
-      <x:c r="E56" s="7" t="s">
+      <x:c r="E56" s="5" t="s">
         <x:v>372</x:v>
       </x:c>
-      <x:c r="F56" s="7" t="s">
+      <x:c r="F56" s="5" t="s">
         <x:v>345</x:v>
       </x:c>
-      <x:c r="G56" s="7" t="s">
+      <x:c r="G56" s="5" t="s">
         <x:v>346</x:v>
       </x:c>
-      <x:c r="H56" s="7" t="s">
+      <x:c r="H56" s="5" t="s">
         <x:v>373</x:v>
       </x:c>
-      <x:c r="I56" s="7" t="s">
+      <x:c r="I56" s="5" t="s">
         <x:v>349</x:v>
       </x:c>
       <x:c r="J56">
@@ -5468,28 +5328,28 @@
       <x:c r="A57">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="B57" s="5" t="s">
+      <x:c r="B57" s="3" t="s">
         <x:v>374</x:v>
       </x:c>
-      <x:c r="C57" s="6">
+      <x:c r="C57" s="4">
         <x:v>45724</x:v>
       </x:c>
-      <x:c r="D57" s="7" t="s">
+      <x:c r="D57" s="5" t="s">
         <x:v>375</x:v>
       </x:c>
-      <x:c r="E57" s="7" t="s">
+      <x:c r="E57" s="5" t="s">
         <x:v>376</x:v>
       </x:c>
-      <x:c r="F57" s="7" t="s">
+      <x:c r="F57" s="5" t="s">
         <x:v>377</x:v>
       </x:c>
-      <x:c r="G57" s="7" t="s">
+      <x:c r="G57" s="5" t="s">
         <x:v>378</x:v>
       </x:c>
-      <x:c r="H57" s="7" t="s">
+      <x:c r="H57" s="5" t="s">
         <x:v>379</x:v>
       </x:c>
-      <x:c r="I57" s="7" t="s">
+      <x:c r="I57" s="5" t="s">
         <x:v>380</x:v>
       </x:c>
       <x:c r="J57">
@@ -5509,28 +5369,28 @@
       <x:c r="A58">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="B58" s="5" t="s">
+      <x:c r="B58" s="3" t="s">
         <x:v>381</x:v>
       </x:c>
-      <x:c r="C58" s="6">
+      <x:c r="C58" s="4">
         <x:v>41107</x:v>
       </x:c>
-      <x:c r="D58" s="7" t="s">
+      <x:c r="D58" s="5" t="s">
         <x:v>382</x:v>
       </x:c>
-      <x:c r="E58" s="7" t="s">
+      <x:c r="E58" s="5" t="s">
         <x:v>383</x:v>
       </x:c>
-      <x:c r="F58" s="7" t="s">
+      <x:c r="F58" s="5" t="s">
         <x:v>384</x:v>
       </x:c>
-      <x:c r="G58" s="7" t="s">
+      <x:c r="G58" s="5" t="s">
         <x:v>385</x:v>
       </x:c>
-      <x:c r="H58" s="7" t="s">
+      <x:c r="H58" s="5" t="s">
         <x:v>386</x:v>
       </x:c>
-      <x:c r="I58" s="7" t="s">
+      <x:c r="I58" s="5" t="s">
         <x:v>387</x:v>
       </x:c>
       <x:c r="J58">
@@ -5550,28 +5410,28 @@
       <x:c r="A59">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="B59" s="5" t="s">
+      <x:c r="B59" s="3" t="s">
         <x:v>388</x:v>
       </x:c>
-      <x:c r="C59" s="6">
+      <x:c r="C59" s="4">
         <x:v>42462</x:v>
       </x:c>
-      <x:c r="D59" s="7" t="s">
+      <x:c r="D59" s="5" t="s">
         <x:v>389</x:v>
       </x:c>
-      <x:c r="E59" s="7" t="s">
+      <x:c r="E59" s="5" t="s">
         <x:v>390</x:v>
       </x:c>
-      <x:c r="F59" s="7" t="s">
+      <x:c r="F59" s="5" t="s">
         <x:v>391</x:v>
       </x:c>
-      <x:c r="G59" s="7" t="s">
+      <x:c r="G59" s="5" t="s">
         <x:v>392</x:v>
       </x:c>
-      <x:c r="H59" s="7" t="s">
+      <x:c r="H59" s="5" t="s">
         <x:v>393</x:v>
       </x:c>
-      <x:c r="I59" s="7" t="s">
+      <x:c r="I59" s="5" t="s">
         <x:v>394</x:v>
       </x:c>
       <x:c r="J59">
@@ -5591,28 +5451,28 @@
       <x:c r="A60">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="B60" s="5" t="s">
+      <x:c r="B60" s="3" t="s">
         <x:v>395</x:v>
       </x:c>
-      <x:c r="C60" s="6">
+      <x:c r="C60" s="4">
         <x:v>41386</x:v>
       </x:c>
-      <x:c r="D60" s="7" t="s">
+      <x:c r="D60" s="5" t="s">
         <x:v>396</x:v>
       </x:c>
-      <x:c r="E60" s="7" t="s">
+      <x:c r="E60" s="5" t="s">
         <x:v>397</x:v>
       </x:c>
-      <x:c r="F60" s="7" t="s">
+      <x:c r="F60" s="5" t="s">
         <x:v>398</x:v>
       </x:c>
-      <x:c r="G60" s="7" t="s">
+      <x:c r="G60" s="5" t="s">
         <x:v>399</x:v>
       </x:c>
-      <x:c r="H60" s="7" t="s">
+      <x:c r="H60" s="5" t="s">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="I60" s="7" t="s">
+      <x:c r="I60" s="5" t="s">
         <x:v>401</x:v>
       </x:c>
       <x:c r="J60">
@@ -5632,28 +5492,28 @@
       <x:c r="A61">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="B61" s="5" t="s">
+      <x:c r="B61" s="3" t="s">
         <x:v>402</x:v>
       </x:c>
-      <x:c r="C61" s="6">
+      <x:c r="C61" s="4">
         <x:v>42904</x:v>
       </x:c>
-      <x:c r="D61" s="7" t="s">
+      <x:c r="D61" s="5" t="s">
         <x:v>403</x:v>
       </x:c>
-      <x:c r="E61" s="7" t="s">
+      <x:c r="E61" s="5" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="F61" s="7" t="s">
+      <x:c r="F61" s="5" t="s">
         <x:v>405</x:v>
       </x:c>
-      <x:c r="G61" s="7" t="s">
+      <x:c r="G61" s="5" t="s">
         <x:v>406</x:v>
       </x:c>
-      <x:c r="H61" s="7" t="s">
+      <x:c r="H61" s="5" t="s">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="I61" s="7" t="s">
+      <x:c r="I61" s="5" t="s">
         <x:v>188</x:v>
       </x:c>
       <x:c r="J61">
@@ -5673,28 +5533,28 @@
       <x:c r="A62">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="B62" s="5" t="s">
+      <x:c r="B62" s="3" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="C62" s="6">
+      <x:c r="C62" s="4">
         <x:v>41130</x:v>
       </x:c>
-      <x:c r="D62" s="7" t="s">
+      <x:c r="D62" s="5" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="E62" s="7" t="s">
+      <x:c r="E62" s="5" t="s">
         <x:v>409</x:v>
       </x:c>
-      <x:c r="F62" s="7" t="s">
+      <x:c r="F62" s="5" t="s">
         <x:v>410</x:v>
       </x:c>
-      <x:c r="G62" s="7" t="s">
+      <x:c r="G62" s="5" t="s">
         <x:v>408</x:v>
       </x:c>
-      <x:c r="H62" s="7" t="s">
+      <x:c r="H62" s="5" t="s">
         <x:v>411</x:v>
       </x:c>
-      <x:c r="I62" s="7" t="s">
+      <x:c r="I62" s="5" t="s">
         <x:v>412</x:v>
       </x:c>
       <x:c r="J62">
@@ -5714,28 +5574,28 @@
       <x:c r="A63">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="B63" s="5" t="s">
+      <x:c r="B63" s="3" t="s">
         <x:v>413</x:v>
       </x:c>
-      <x:c r="C63" s="6">
+      <x:c r="C63" s="4">
         <x:v>41487</x:v>
       </x:c>
-      <x:c r="D63" s="7" t="s">
+      <x:c r="D63" s="5" t="s">
         <x:v>414</x:v>
       </x:c>
-      <x:c r="E63" s="7" t="s">
+      <x:c r="E63" s="5" t="s">
         <x:v>415</x:v>
       </x:c>
-      <x:c r="F63" s="7" t="s">
+      <x:c r="F63" s="5" t="s">
         <x:v>416</x:v>
       </x:c>
-      <x:c r="G63" s="7" t="s">
+      <x:c r="G63" s="5" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="H63" s="7" t="s">
+      <x:c r="H63" s="5" t="s">
         <x:v>417</x:v>
       </x:c>
-      <x:c r="I63" s="7" t="s">
+      <x:c r="I63" s="5" t="s">
         <x:v>418</x:v>
       </x:c>
       <x:c r="J63">
@@ -5755,28 +5615,28 @@
       <x:c r="A64">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="B64" s="5" t="s">
+      <x:c r="B64" s="3" t="s">
         <x:v>419</x:v>
       </x:c>
-      <x:c r="C64" s="6">
+      <x:c r="C64" s="4">
         <x:v>41108</x:v>
       </x:c>
-      <x:c r="D64" s="7" t="s">
+      <x:c r="D64" s="5" t="s">
         <x:v>420</x:v>
       </x:c>
-      <x:c r="E64" s="7" t="s">
+      <x:c r="E64" s="5" t="s">
         <x:v>421</x:v>
       </x:c>
-      <x:c r="F64" s="7" t="s">
+      <x:c r="F64" s="5" t="s">
         <x:v>422</x:v>
       </x:c>
-      <x:c r="G64" s="7" t="s">
+      <x:c r="G64" s="5" t="s">
         <x:v>423</x:v>
       </x:c>
-      <x:c r="H64" s="7" t="s">
+      <x:c r="H64" s="5" t="s">
         <x:v>424</x:v>
       </x:c>
-      <x:c r="I64" s="7" t="s">
+      <x:c r="I64" s="5" t="s">
         <x:v>425</x:v>
       </x:c>
       <x:c r="J64">
@@ -5796,28 +5656,28 @@
       <x:c r="A65">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="B65" s="5" t="s">
+      <x:c r="B65" s="3" t="s">
         <x:v>426</x:v>
       </x:c>
-      <x:c r="C65" s="6">
+      <x:c r="C65" s="4">
         <x:v>43586</x:v>
       </x:c>
-      <x:c r="D65" s="7" t="s">
+      <x:c r="D65" s="5" t="s">
         <x:v>427</x:v>
       </x:c>
-      <x:c r="E65" s="7" t="s">
+      <x:c r="E65" s="5" t="s">
         <x:v>428</x:v>
       </x:c>
-      <x:c r="F65" s="7" t="s">
+      <x:c r="F65" s="5" t="s">
         <x:v>429</x:v>
       </x:c>
-      <x:c r="G65" s="7" t="s">
+      <x:c r="G65" s="5" t="s">
         <x:v>430</x:v>
       </x:c>
-      <x:c r="H65" s="7" t="s">
+      <x:c r="H65" s="5" t="s">
         <x:v>431</x:v>
       </x:c>
-      <x:c r="I65" s="7" t="s">
+      <x:c r="I65" s="5" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="J65">
@@ -5837,28 +5697,28 @@
       <x:c r="A66">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="B66" s="5" t="s">
+      <x:c r="B66" s="3" t="s">
         <x:v>433</x:v>
       </x:c>
-      <x:c r="C66" s="6">
+      <x:c r="C66" s="4">
         <x:v>42753</x:v>
       </x:c>
-      <x:c r="D66" s="7" t="s">
+      <x:c r="D66" s="5" t="s">
         <x:v>434</x:v>
       </x:c>
-      <x:c r="E66" s="7" t="s">
+      <x:c r="E66" s="5" t="s">
         <x:v>435</x:v>
       </x:c>
-      <x:c r="F66" s="7" t="s">
+      <x:c r="F66" s="5" t="s">
         <x:v>436</x:v>
       </x:c>
-      <x:c r="G66" s="7" t="s">
+      <x:c r="G66" s="5" t="s">
         <x:v>437</x:v>
       </x:c>
-      <x:c r="H66" s="7" t="s">
+      <x:c r="H66" s="5" t="s">
         <x:v>438</x:v>
       </x:c>
-      <x:c r="I66" s="7" t="s">
+      <x:c r="I66" s="5" t="s">
         <x:v>439</x:v>
       </x:c>
       <x:c r="J66">
@@ -5878,28 +5738,28 @@
       <x:c r="A67">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="B67" s="5" t="s">
+      <x:c r="B67" s="3" t="s">
         <x:v>440</x:v>
       </x:c>
-      <x:c r="C67" s="6">
+      <x:c r="C67" s="4">
         <x:v>41113</x:v>
       </x:c>
-      <x:c r="D67" s="7" t="s">
+      <x:c r="D67" s="5" t="s">
         <x:v>441</x:v>
       </x:c>
-      <x:c r="E67" s="7" t="s">
+      <x:c r="E67" s="5" t="s">
         <x:v>442</x:v>
       </x:c>
-      <x:c r="F67" s="7" t="s">
+      <x:c r="F67" s="5" t="s">
         <x:v>443</x:v>
       </x:c>
-      <x:c r="G67" s="7" t="s">
+      <x:c r="G67" s="5" t="s">
         <x:v>444</x:v>
       </x:c>
-      <x:c r="H67" s="7" t="s">
+      <x:c r="H67" s="5" t="s">
         <x:v>445</x:v>
       </x:c>
-      <x:c r="I67" s="7" t="s">
+      <x:c r="I67" s="5" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="J67">
@@ -5919,28 +5779,28 @@
       <x:c r="A68">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="B68" s="5" t="s">
+      <x:c r="B68" s="3" t="s">
         <x:v>447</x:v>
       </x:c>
-      <x:c r="C68" s="6">
+      <x:c r="C68" s="4">
         <x:v>42177</x:v>
       </x:c>
-      <x:c r="D68" s="7" t="s">
+      <x:c r="D68" s="5" t="s">
         <x:v>448</x:v>
       </x:c>
-      <x:c r="E68" s="7" t="s">
+      <x:c r="E68" s="5" t="s">
         <x:v>449</x:v>
       </x:c>
-      <x:c r="F68" s="7" t="s">
+      <x:c r="F68" s="5" t="s">
         <x:v>450</x:v>
       </x:c>
-      <x:c r="G68" s="7" t="s">
+      <x:c r="G68" s="5" t="s">
         <x:v>451</x:v>
       </x:c>
-      <x:c r="H68" s="7" t="s">
+      <x:c r="H68" s="5" t="s">
         <x:v>452</x:v>
       </x:c>
-      <x:c r="I68" s="7" t="s">
+      <x:c r="I68" s="5" t="s">
         <x:v>453</x:v>
       </x:c>
       <x:c r="J68">
@@ -5960,28 +5820,28 @@
       <x:c r="A69">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="B69" s="5" t="s">
+      <x:c r="B69" s="3" t="s">
         <x:v>454</x:v>
       </x:c>
-      <x:c r="C69" s="6">
+      <x:c r="C69" s="4">
         <x:v>41712</x:v>
       </x:c>
-      <x:c r="D69" s="7" t="s">
+      <x:c r="D69" s="5" t="s">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="E69" s="7" t="s">
+      <x:c r="E69" s="5" t="s">
         <x:v>456</x:v>
       </x:c>
-      <x:c r="F69" s="7" t="s">
+      <x:c r="F69" s="5" t="s">
         <x:v>457</x:v>
       </x:c>
-      <x:c r="G69" s="7" t="s">
+      <x:c r="G69" s="5" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="H69" s="7" t="s">
+      <x:c r="H69" s="5" t="s">
         <x:v>458</x:v>
       </x:c>
-      <x:c r="I69" s="7" t="s">
+      <x:c r="I69" s="5" t="s">
         <x:v>459</x:v>
       </x:c>
       <x:c r="J69">
@@ -6001,29 +5861,29 @@
       <x:c r="A70">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="B70" s="5" t="s">
+      <x:c r="B70" s="3" t="s">
         <x:v>460</x:v>
       </x:c>
-      <x:c r="C70" s="6">
+      <x:c r="C70" s="4">
         <x:v>43013</x:v>
       </x:c>
-      <x:c r="D70" s="7" t="s">
+      <x:c r="D70" s="5" t="s">
         <x:v>461</x:v>
       </x:c>
-      <x:c r="E70" s="7" t="s">
+      <x:c r="E70" s="5" t="s">
         <x:v>462</x:v>
       </x:c>
-      <x:c r="F70" s="7" t="s">
+      <x:c r="F70" s="5" t="s">
         <x:v>463</x:v>
       </x:c>
-      <x:c r="G70" s="7" t="s">
+      <x:c r="G70" s="5" t="s">
         <x:v>464</x:v>
       </x:c>
-      <x:c r="H70" s="7" t="s">
+      <x:c r="H70" s="5" t="s">
         <x:v>465</x:v>
       </x:c>
-      <x:c r="I70" s="7" t="str">
-        <x:v>我唱人间</x:v>
+      <x:c r="I70" s="5" t="s">
+        <x:v>466</x:v>
       </x:c>
       <x:c r="J70">
         <x:v>11</x:v>
@@ -6042,29 +5902,29 @@
       <x:c r="A71">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="B71" s="5" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="C71" s="6">
+      <x:c r="B71" s="3" t="s">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="C71" s="4">
         <x:v>43364</x:v>
       </x:c>
-      <x:c r="D71" s="7" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="E71" s="7" t="s">
+      <x:c r="D71" s="5" t="s">
         <x:v>468</x:v>
       </x:c>
-      <x:c r="F71" s="7" t="s">
+      <x:c r="E71" s="5" t="s">
         <x:v>469</x:v>
       </x:c>
-      <x:c r="G71" s="7" t="s">
+      <x:c r="F71" s="5" t="s">
         <x:v>470</x:v>
       </x:c>
-      <x:c r="H71" s="7" t="s">
+      <x:c r="G71" s="5" t="s">
         <x:v>471</x:v>
       </x:c>
-      <x:c r="I71" s="7" t="s">
+      <x:c r="H71" s="5" t="s">
         <x:v>472</x:v>
+      </x:c>
+      <x:c r="I71" s="5" t="s">
+        <x:v>473</x:v>
       </x:c>
       <x:c r="J71">
         <x:v>9</x:v>
@@ -6083,29 +5943,29 @@
       <x:c r="A72">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="B72" s="5" t="s">
-        <x:v>473</x:v>
-      </x:c>
-      <x:c r="C72" s="6">
+      <x:c r="B72" s="3" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="C72" s="4">
         <x:v>41110</x:v>
       </x:c>
-      <x:c r="D72" s="7" t="s">
-        <x:v>474</x:v>
-      </x:c>
-      <x:c r="E72" s="7" t="s">
+      <x:c r="D72" s="5" t="s">
         <x:v>475</x:v>
       </x:c>
-      <x:c r="F72" s="7" t="s">
+      <x:c r="E72" s="5" t="s">
         <x:v>476</x:v>
       </x:c>
-      <x:c r="G72" s="7" t="s">
+      <x:c r="F72" s="5" t="s">
         <x:v>477</x:v>
       </x:c>
-      <x:c r="H72" s="7" t="s">
+      <x:c r="G72" s="5" t="s">
         <x:v>478</x:v>
       </x:c>
-      <x:c r="I72" s="7" t="s">
+      <x:c r="H72" s="5" t="s">
         <x:v>479</x:v>
+      </x:c>
+      <x:c r="I72" s="5" t="s">
+        <x:v>480</x:v>
       </x:c>
       <x:c r="J72">
         <x:v>86</x:v>
@@ -6124,29 +5984,29 @@
       <x:c r="A73">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="B73" s="5" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="C73" s="6">
+      <x:c r="B73" s="3" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="C73" s="4">
         <x:v>42228</x:v>
       </x:c>
-      <x:c r="D73" s="7" t="s">
-        <x:v>481</x:v>
-      </x:c>
-      <x:c r="E73" s="7" t="s">
+      <x:c r="D73" s="5" t="s">
         <x:v>482</x:v>
       </x:c>
-      <x:c r="F73" s="7" t="s">
+      <x:c r="E73" s="5" t="s">
         <x:v>483</x:v>
       </x:c>
-      <x:c r="G73" s="7" t="s">
+      <x:c r="F73" s="5" t="s">
         <x:v>484</x:v>
       </x:c>
-      <x:c r="H73" s="7" t="s">
+      <x:c r="G73" s="5" t="s">
         <x:v>485</x:v>
       </x:c>
-      <x:c r="I73" s="7" t="s">
+      <x:c r="H73" s="5" t="s">
         <x:v>486</x:v>
+      </x:c>
+      <x:c r="I73" s="5" t="s">
+        <x:v>487</x:v>
       </x:c>
       <x:c r="J73">
         <x:v>11</x:v>
@@ -6165,29 +6025,29 @@
       <x:c r="A74">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="B74" s="5" t="s">
-        <x:v>487</x:v>
-      </x:c>
-      <x:c r="C74" s="6">
+      <x:c r="B74" s="3" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="C74" s="4">
         <x:v>41174</x:v>
       </x:c>
-      <x:c r="D74" s="7" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E74" s="7" t="s">
+      <x:c r="D74" s="5" t="s">
         <x:v>489</x:v>
       </x:c>
-      <x:c r="F74" s="7" t="s">
+      <x:c r="E74" s="5" t="s">
         <x:v>490</x:v>
       </x:c>
-      <x:c r="G74" s="7" t="s">
+      <x:c r="F74" s="5" t="s">
         <x:v>491</x:v>
       </x:c>
-      <x:c r="H74" s="7" t="s">
+      <x:c r="G74" s="5" t="s">
         <x:v>492</x:v>
       </x:c>
-      <x:c r="I74" s="7" t="s">
+      <x:c r="H74" s="5" t="s">
         <x:v>493</x:v>
+      </x:c>
+      <x:c r="I74" s="5" t="s">
+        <x:v>494</x:v>
       </x:c>
       <x:c r="J74">
         <x:v>5</x:v>
@@ -6206,29 +6066,29 @@
       <x:c r="A75">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="B75" s="5" t="s">
-        <x:v>494</x:v>
-      </x:c>
-      <x:c r="C75" s="6">
+      <x:c r="B75" s="3" t="s">
+        <x:v>495</x:v>
+      </x:c>
+      <x:c r="C75" s="4">
         <x:v>41542</x:v>
       </x:c>
-      <x:c r="D75" s="7" t="s">
-        <x:v>495</x:v>
-      </x:c>
-      <x:c r="E75" s="7" t="s">
+      <x:c r="D75" s="5" t="s">
         <x:v>496</x:v>
       </x:c>
-      <x:c r="F75" s="7" t="s">
+      <x:c r="E75" s="5" t="s">
         <x:v>497</x:v>
       </x:c>
-      <x:c r="G75" s="7" t="s">
+      <x:c r="F75" s="5" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="H75" s="7" t="s">
+      <x:c r="G75" s="5" t="s">
         <x:v>499</x:v>
       </x:c>
-      <x:c r="I75" s="7" t="s">
+      <x:c r="H75" s="5" t="s">
         <x:v>500</x:v>
+      </x:c>
+      <x:c r="I75" s="5" t="s">
+        <x:v>501</x:v>
       </x:c>
       <x:c r="J75">
         <x:v>20</x:v>
@@ -6247,29 +6107,29 @@
       <x:c r="A76">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="B76" s="5" t="s">
-        <x:v>501</x:v>
-      </x:c>
-      <x:c r="C76" s="6">
+      <x:c r="B76" s="3" t="s">
+        <x:v>502</x:v>
+      </x:c>
+      <x:c r="C76" s="4">
         <x:v>42152</x:v>
       </x:c>
-      <x:c r="D76" s="7" t="s">
-        <x:v>502</x:v>
-      </x:c>
-      <x:c r="E76" s="7" t="s">
+      <x:c r="D76" s="5" t="s">
         <x:v>503</x:v>
       </x:c>
-      <x:c r="F76" s="7" t="s">
+      <x:c r="E76" s="5" t="s">
         <x:v>504</x:v>
       </x:c>
-      <x:c r="G76" s="7" t="s">
+      <x:c r="F76" s="5" t="s">
         <x:v>505</x:v>
       </x:c>
-      <x:c r="H76" s="7" t="s">
+      <x:c r="G76" s="5" t="s">
         <x:v>506</x:v>
       </x:c>
-      <x:c r="I76" s="7" t="s">
+      <x:c r="H76" s="5" t="s">
         <x:v>507</x:v>
+      </x:c>
+      <x:c r="I76" s="5" t="s">
+        <x:v>508</x:v>
       </x:c>
       <x:c r="J76">
         <x:v>10</x:v>
@@ -6288,29 +6148,29 @@
       <x:c r="A77">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="B77" s="5" t="s">
-        <x:v>508</x:v>
-      </x:c>
-      <x:c r="C77" s="6">
+      <x:c r="B77" s="3" t="s">
+        <x:v>509</x:v>
+      </x:c>
+      <x:c r="C77" s="4">
         <x:v>45143</x:v>
       </x:c>
-      <x:c r="D77" s="7" t="s">
-        <x:v>509</x:v>
-      </x:c>
-      <x:c r="E77" s="7" t="s">
+      <x:c r="D77" s="5" t="s">
         <x:v>510</x:v>
       </x:c>
-      <x:c r="F77" s="7" t="s">
+      <x:c r="E77" s="5" t="s">
         <x:v>511</x:v>
       </x:c>
-      <x:c r="G77" s="7" t="s">
+      <x:c r="F77" s="5" t="s">
         <x:v>512</x:v>
       </x:c>
-      <x:c r="H77" s="7" t="s">
+      <x:c r="G77" s="5" t="s">
         <x:v>513</x:v>
       </x:c>
-      <x:c r="I77" s="7" t="s">
+      <x:c r="H77" s="5" t="s">
         <x:v>514</x:v>
+      </x:c>
+      <x:c r="I77" s="5" t="s">
+        <x:v>515</x:v>
       </x:c>
       <x:c r="J77">
         <x:v>10</x:v>
@@ -6329,29 +6189,29 @@
       <x:c r="A78">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="B78" s="5" t="s">
-        <x:v>515</x:v>
-      </x:c>
-      <x:c r="C78" s="6">
+      <x:c r="B78" s="3" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="C78" s="4">
         <x:v>41614</x:v>
       </x:c>
-      <x:c r="D78" s="7" t="s">
-        <x:v>516</x:v>
-      </x:c>
-      <x:c r="E78" s="7" t="s">
+      <x:c r="D78" s="5" t="s">
         <x:v>517</x:v>
       </x:c>
-      <x:c r="F78" s="7" t="s">
-        <x:v>516</x:v>
-      </x:c>
-      <x:c r="G78" s="7" t="s">
+      <x:c r="E78" s="5" t="s">
         <x:v>518</x:v>
       </x:c>
-      <x:c r="H78" s="7" t="s">
+      <x:c r="F78" s="5" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="G78" s="5" t="s">
         <x:v>519</x:v>
       </x:c>
-      <x:c r="I78" s="7" t="s">
+      <x:c r="H78" s="5" t="s">
         <x:v>520</x:v>
+      </x:c>
+      <x:c r="I78" s="5" t="s">
+        <x:v>521</x:v>
       </x:c>
       <x:c r="J78">
         <x:v>8</x:v>
@@ -6370,29 +6230,29 @@
       <x:c r="A79">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="B79" s="5" t="s">
-        <x:v>521</x:v>
-      </x:c>
-      <x:c r="C79" s="6">
+      <x:c r="B79" s="3" t="s">
+        <x:v>522</x:v>
+      </x:c>
+      <x:c r="C79" s="4">
         <x:v>43154</x:v>
       </x:c>
-      <x:c r="D79" s="7" t="s">
-        <x:v>522</x:v>
-      </x:c>
-      <x:c r="E79" s="7" t="s">
+      <x:c r="D79" s="5" t="s">
         <x:v>523</x:v>
       </x:c>
-      <x:c r="F79" s="7" t="s">
+      <x:c r="E79" s="5" t="s">
         <x:v>524</x:v>
       </x:c>
-      <x:c r="G79" s="7" t="s">
+      <x:c r="F79" s="5" t="s">
         <x:v>525</x:v>
       </x:c>
-      <x:c r="H79" s="7" t="s">
+      <x:c r="G79" s="5" t="s">
         <x:v>526</x:v>
       </x:c>
-      <x:c r="I79" s="7" t="s">
+      <x:c r="H79" s="5" t="s">
         <x:v>527</x:v>
+      </x:c>
+      <x:c r="I79" s="5" t="s">
+        <x:v>528</x:v>
       </x:c>
       <x:c r="J79">
         <x:v>4</x:v>
@@ -6411,29 +6271,29 @@
       <x:c r="A80">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="B80" s="5" t="s">
-        <x:v>528</x:v>
-      </x:c>
-      <x:c r="C80" s="6">
+      <x:c r="B80" s="3" t="s">
+        <x:v>529</x:v>
+      </x:c>
+      <x:c r="C80" s="4">
         <x:v>45131</x:v>
       </x:c>
-      <x:c r="D80" s="7" t="s">
-        <x:v>529</x:v>
-      </x:c>
-      <x:c r="E80" s="7" t="s">
+      <x:c r="D80" s="5" t="s">
         <x:v>530</x:v>
       </x:c>
-      <x:c r="F80" s="7" t="s">
+      <x:c r="E80" s="5" t="s">
         <x:v>531</x:v>
       </x:c>
-      <x:c r="G80" s="7" t="s">
+      <x:c r="F80" s="5" t="s">
         <x:v>532</x:v>
       </x:c>
-      <x:c r="H80" s="7" t="s">
+      <x:c r="G80" s="5" t="s">
         <x:v>533</x:v>
       </x:c>
-      <x:c r="I80" s="7" t="s">
+      <x:c r="H80" s="5" t="s">
         <x:v>534</x:v>
+      </x:c>
+      <x:c r="I80" s="5" t="s">
+        <x:v>535</x:v>
       </x:c>
       <x:c r="J80">
         <x:v>1</x:v>
@@ -6444,37 +6304,37 @@
       <x:c r="L80">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M80">
-        <x:v>1</x:v>
+      <x:c r="M80" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="18.75">
       <x:c r="A81">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="B81" s="5" t="s">
-        <x:v>535</x:v>
-      </x:c>
-      <x:c r="C81" s="6">
+      <x:c r="B81" s="3" t="s">
+        <x:v>536</x:v>
+      </x:c>
+      <x:c r="C81" s="4">
         <x:v>41159</x:v>
       </x:c>
-      <x:c r="D81" s="7" t="s">
-        <x:v>536</x:v>
-      </x:c>
-      <x:c r="E81" s="7" t="s">
+      <x:c r="D81" s="5" t="s">
+        <x:v>537</x:v>
+      </x:c>
+      <x:c r="E81" s="5" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="F81" s="7" t="s">
-        <x:v>537</x:v>
-      </x:c>
-      <x:c r="G81" s="7" t="s">
+      <x:c r="F81" s="5" t="s">
         <x:v>538</x:v>
       </x:c>
-      <x:c r="H81" s="7" t="s">
+      <x:c r="G81" s="5" t="s">
         <x:v>539</x:v>
       </x:c>
-      <x:c r="I81" s="7" t="s">
+      <x:c r="H81" s="5" t="s">
         <x:v>540</x:v>
+      </x:c>
+      <x:c r="I81" s="5" t="s">
+        <x:v>541</x:v>
       </x:c>
       <x:c r="J81">
         <x:v>12</x:v>
@@ -6493,29 +6353,29 @@
       <x:c r="A82">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="B82" s="5" t="s">
-        <x:v>541</x:v>
-      </x:c>
-      <x:c r="C82" s="6">
+      <x:c r="B82" s="3" t="s">
+        <x:v>542</x:v>
+      </x:c>
+      <x:c r="C82" s="4">
         <x:v>43777</x:v>
       </x:c>
-      <x:c r="D82" s="7" t="s">
-        <x:v>542</x:v>
-      </x:c>
-      <x:c r="E82" s="7" t="s">
+      <x:c r="D82" s="5" t="s">
         <x:v>543</x:v>
       </x:c>
-      <x:c r="F82" s="7" t="s">
+      <x:c r="E82" s="5" t="s">
         <x:v>544</x:v>
       </x:c>
-      <x:c r="G82" s="7" t="s">
+      <x:c r="F82" s="5" t="s">
         <x:v>545</x:v>
       </x:c>
-      <x:c r="H82" s="7" t="s">
+      <x:c r="G82" s="5" t="s">
         <x:v>546</x:v>
       </x:c>
-      <x:c r="I82" s="7" t="s">
+      <x:c r="H82" s="5" t="s">
         <x:v>547</x:v>
+      </x:c>
+      <x:c r="I82" s="5" t="s">
+        <x:v>548</x:v>
       </x:c>
       <x:c r="J82">
         <x:v>22</x:v>
@@ -6534,29 +6394,29 @@
       <x:c r="A83">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="B83" s="5" t="s">
-        <x:v>548</x:v>
-      </x:c>
-      <x:c r="C83" s="6">
+      <x:c r="B83" s="3" t="s">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="C83" s="4">
         <x:v>41521</x:v>
       </x:c>
-      <x:c r="D83" s="7" t="s">
-        <x:v>549</x:v>
-      </x:c>
-      <x:c r="E83" s="7" t="s">
+      <x:c r="D83" s="5" t="s">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="E83" s="5" t="s">
         <x:v>456</x:v>
       </x:c>
-      <x:c r="F83" s="7" t="s">
+      <x:c r="F83" s="5" t="s">
         <x:v>195</x:v>
       </x:c>
-      <x:c r="G83" s="7" t="s">
+      <x:c r="G83" s="5" t="s">
         <x:v>397</x:v>
       </x:c>
-      <x:c r="H83" s="7" t="s">
+      <x:c r="H83" s="5" t="s">
         <x:v>457</x:v>
       </x:c>
-      <x:c r="I83" s="7" t="s">
-        <x:v>550</x:v>
+      <x:c r="I83" s="5" t="s">
+        <x:v>551</x:v>
       </x:c>
       <x:c r="J83">
         <x:v>26</x:v>
@@ -6575,29 +6435,29 @@
       <x:c r="A84">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="B84" s="5" t="s">
-        <x:v>551</x:v>
-      </x:c>
-      <x:c r="C84" s="6">
+      <x:c r="B84" s="3" t="s">
+        <x:v>552</x:v>
+      </x:c>
+      <x:c r="C84" s="4">
         <x:v>45632</x:v>
       </x:c>
-      <x:c r="D84" s="7" t="s">
-        <x:v>552</x:v>
-      </x:c>
-      <x:c r="E84" s="7" t="s">
+      <x:c r="D84" s="5" t="s">
         <x:v>553</x:v>
       </x:c>
-      <x:c r="F84" s="7" t="s">
+      <x:c r="E84" s="5" t="s">
         <x:v>554</x:v>
       </x:c>
-      <x:c r="G84" s="7" t="s">
+      <x:c r="F84" s="5" t="s">
         <x:v>555</x:v>
       </x:c>
-      <x:c r="H84" s="7" t="s">
+      <x:c r="G84" s="5" t="s">
         <x:v>556</x:v>
       </x:c>
-      <x:c r="I84" s="7" t="s">
+      <x:c r="H84" s="5" t="s">
         <x:v>557</x:v>
+      </x:c>
+      <x:c r="I84" s="5" t="s">
+        <x:v>558</x:v>
       </x:c>
       <x:c r="J84">
         <x:v>4</x:v>
@@ -6616,29 +6476,29 @@
       <x:c r="A85">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="B85" s="5" t="s">
-        <x:v>558</x:v>
-      </x:c>
-      <x:c r="C85" s="6">
+      <x:c r="B85" s="3" t="s">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c r="C85" s="4">
         <x:v>42195</x:v>
       </x:c>
-      <x:c r="D85" s="7" t="s">
-        <x:v>559</x:v>
-      </x:c>
-      <x:c r="E85" s="7" t="s">
+      <x:c r="D85" s="5" t="s">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="E85" s="5" t="s">
         <x:v>399</x:v>
       </x:c>
-      <x:c r="F85" s="7" t="s">
+      <x:c r="F85" s="5" t="s">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="G85" s="7" t="s">
-        <x:v>559</x:v>
-      </x:c>
-      <x:c r="H85" s="7" t="s">
+      <x:c r="G85" s="5" t="s">
         <x:v>560</x:v>
       </x:c>
-      <x:c r="I85" s="7" t="s">
+      <x:c r="H85" s="5" t="s">
         <x:v>561</x:v>
+      </x:c>
+      <x:c r="I85" s="5" t="s">
+        <x:v>562</x:v>
       </x:c>
       <x:c r="J85">
         <x:v>9</x:v>
@@ -6657,29 +6517,29 @@
       <x:c r="A86">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B86" s="5" t="s">
-        <x:v>562</x:v>
-      </x:c>
-      <x:c r="C86" s="6">
+      <x:c r="B86" s="3" t="s">
+        <x:v>563</x:v>
+      </x:c>
+      <x:c r="C86" s="4">
         <x:v>41291</x:v>
       </x:c>
-      <x:c r="D86" s="7" t="s">
-        <x:v>563</x:v>
-      </x:c>
-      <x:c r="E86" s="7" t="s">
+      <x:c r="D86" s="5" t="s">
         <x:v>564</x:v>
       </x:c>
-      <x:c r="F86" s="7" t="s">
+      <x:c r="E86" s="5" t="s">
         <x:v>565</x:v>
       </x:c>
-      <x:c r="G86" s="7" t="s">
+      <x:c r="F86" s="5" t="s">
         <x:v>566</x:v>
       </x:c>
-      <x:c r="H86" s="7" t="s">
+      <x:c r="G86" s="5" t="s">
         <x:v>567</x:v>
       </x:c>
-      <x:c r="I86" s="7" t="s">
+      <x:c r="H86" s="5" t="s">
         <x:v>568</x:v>
+      </x:c>
+      <x:c r="I86" s="5" t="s">
+        <x:v>569</x:v>
       </x:c>
       <x:c r="J86">
         <x:v>19</x:v>
@@ -6698,29 +6558,29 @@
       <x:c r="A87">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="B87" s="5" t="s">
-        <x:v>569</x:v>
-      </x:c>
-      <x:c r="C87" s="6">
+      <x:c r="B87" s="3" t="s">
+        <x:v>570</x:v>
+      </x:c>
+      <x:c r="C87" s="4">
         <x:v>41377</x:v>
       </x:c>
-      <x:c r="D87" s="7" t="s">
-        <x:v>570</x:v>
-      </x:c>
-      <x:c r="E87" s="7" t="s">
+      <x:c r="D87" s="5" t="s">
         <x:v>571</x:v>
       </x:c>
-      <x:c r="F87" s="7" t="s">
+      <x:c r="E87" s="5" t="s">
         <x:v>572</x:v>
       </x:c>
-      <x:c r="G87" s="7" t="s">
+      <x:c r="F87" s="5" t="s">
         <x:v>573</x:v>
       </x:c>
-      <x:c r="H87" s="7" t="s">
+      <x:c r="G87" s="5" t="s">
         <x:v>574</x:v>
       </x:c>
-      <x:c r="I87" s="7" t="s">
+      <x:c r="H87" s="5" t="s">
         <x:v>575</x:v>
+      </x:c>
+      <x:c r="I87" s="5" t="s">
+        <x:v>576</x:v>
       </x:c>
       <x:c r="J87">
         <x:v>9</x:v>
@@ -6739,29 +6599,29 @@
       <x:c r="A88">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="B88" s="5" t="s">
-        <x:v>576</x:v>
-      </x:c>
-      <x:c r="C88" s="6">
+      <x:c r="B88" s="3" t="s">
+        <x:v>577</x:v>
+      </x:c>
+      <x:c r="C88" s="4">
         <x:v>43378</x:v>
       </x:c>
-      <x:c r="D88" s="7" t="s">
-        <x:v>577</x:v>
-      </x:c>
-      <x:c r="E88" s="7" t="s">
+      <x:c r="D88" s="5" t="s">
         <x:v>578</x:v>
       </x:c>
-      <x:c r="F88" s="7" t="s">
+      <x:c r="E88" s="5" t="s">
         <x:v>579</x:v>
       </x:c>
-      <x:c r="G88" s="7" t="s">
+      <x:c r="F88" s="5" t="s">
         <x:v>580</x:v>
       </x:c>
-      <x:c r="H88" s="7" t="s">
+      <x:c r="G88" s="5" t="s">
         <x:v>581</x:v>
       </x:c>
-      <x:c r="I88" s="7" t="s">
+      <x:c r="H88" s="5" t="s">
         <x:v>582</x:v>
+      </x:c>
+      <x:c r="I88" s="5" t="s">
+        <x:v>583</x:v>
       </x:c>
       <x:c r="J88">
         <x:v>10</x:v>
@@ -6780,29 +6640,29 @@
       <x:c r="A89">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="B89" s="5" t="s">
-        <x:v>583</x:v>
-      </x:c>
-      <x:c r="C89" s="6">
+      <x:c r="B89" s="3" t="s">
+        <x:v>584</x:v>
+      </x:c>
+      <x:c r="C89" s="4">
         <x:v>41327</x:v>
       </x:c>
-      <x:c r="D89" s="7" t="s">
-        <x:v>584</x:v>
-      </x:c>
-      <x:c r="E89" s="7" t="s">
+      <x:c r="D89" s="5" t="s">
         <x:v>585</x:v>
       </x:c>
-      <x:c r="F89" s="7" t="s">
+      <x:c r="E89" s="5" t="s">
         <x:v>586</x:v>
       </x:c>
-      <x:c r="G89" s="7" t="s">
+      <x:c r="F89" s="5" t="s">
         <x:v>587</x:v>
       </x:c>
-      <x:c r="H89" s="7" t="s">
+      <x:c r="G89" s="5" t="s">
+        <x:v>588</x:v>
+      </x:c>
+      <x:c r="H89" s="5" t="s">
         <x:v>209</x:v>
       </x:c>
-      <x:c r="I89" s="7" t="s">
-        <x:v>588</x:v>
+      <x:c r="I89" s="5" t="s">
+        <x:v>589</x:v>
       </x:c>
       <x:c r="J89">
         <x:v>33</x:v>
@@ -6821,28 +6681,28 @@
       <x:c r="A90">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="B90" s="5" t="s">
-        <x:v>589</x:v>
-      </x:c>
-      <x:c r="C90" s="6">
+      <x:c r="B90" s="3" t="s">
+        <x:v>590</x:v>
+      </x:c>
+      <x:c r="C90" s="4">
         <x:v>41122</x:v>
       </x:c>
-      <x:c r="D90" s="7" t="s">
-        <x:v>590</x:v>
-      </x:c>
-      <x:c r="E90" s="7" t="s">
+      <x:c r="D90" s="5" t="s">
+        <x:v>591</x:v>
+      </x:c>
+      <x:c r="E90" s="5" t="s">
         <x:v>443</x:v>
       </x:c>
-      <x:c r="F90" s="7" t="s">
-        <x:v>591</x:v>
-      </x:c>
-      <x:c r="G90" s="7" t="s">
+      <x:c r="F90" s="5" t="s">
+        <x:v>592</x:v>
+      </x:c>
+      <x:c r="G90" s="5" t="s">
         <x:v>421</x:v>
       </x:c>
-      <x:c r="H90" s="7" t="s">
-        <x:v>592</x:v>
-      </x:c>
-      <x:c r="I90" s="7" t="s">
+      <x:c r="H90" s="5" t="s">
+        <x:v>593</x:v>
+      </x:c>
+      <x:c r="I90" s="5" t="s">
         <x:v>423</x:v>
       </x:c>
       <x:c r="J90">
@@ -6862,29 +6722,29 @@
       <x:c r="A91">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B91" s="5" t="s">
-        <x:v>593</x:v>
-      </x:c>
-      <x:c r="C91" s="6">
+      <x:c r="B91" s="3" t="s">
+        <x:v>594</x:v>
+      </x:c>
+      <x:c r="C91" s="4">
         <x:v>42356</x:v>
       </x:c>
-      <x:c r="D91" s="7" t="s">
-        <x:v>594</x:v>
-      </x:c>
-      <x:c r="E91" s="7" t="s">
+      <x:c r="D91" s="5" t="s">
         <x:v>595</x:v>
       </x:c>
-      <x:c r="F91" s="7" t="s">
+      <x:c r="E91" s="5" t="s">
         <x:v>596</x:v>
       </x:c>
-      <x:c r="G91" s="7" t="s">
+      <x:c r="F91" s="5" t="s">
         <x:v>597</x:v>
       </x:c>
-      <x:c r="H91" s="7" t="s">
+      <x:c r="G91" s="5" t="s">
         <x:v>598</x:v>
       </x:c>
-      <x:c r="I91" s="7" t="s">
+      <x:c r="H91" s="5" t="s">
         <x:v>599</x:v>
+      </x:c>
+      <x:c r="I91" s="5" t="s">
+        <x:v>600</x:v>
       </x:c>
       <x:c r="J91">
         <x:v>18</x:v>
@@ -6903,29 +6763,29 @@
       <x:c r="A92">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="B92" s="5" t="s">
-        <x:v>600</x:v>
-      </x:c>
-      <x:c r="C92" s="6">
+      <x:c r="B92" s="3" t="s">
+        <x:v>601</x:v>
+      </x:c>
+      <x:c r="C92" s="4">
         <x:v>43074</x:v>
       </x:c>
-      <x:c r="D92" s="7" t="s">
-        <x:v>601</x:v>
-      </x:c>
-      <x:c r="E92" s="7" t="s">
+      <x:c r="D92" s="5" t="s">
+        <x:v>602</x:v>
+      </x:c>
+      <x:c r="E92" s="5" t="s">
         <x:v>463</x:v>
       </x:c>
-      <x:c r="F92" s="7" t="s">
-        <x:v>602</x:v>
-      </x:c>
-      <x:c r="G92" s="7" t="s">
+      <x:c r="F92" s="5" t="s">
         <x:v>603</x:v>
       </x:c>
-      <x:c r="H92" s="7" t="s">
+      <x:c r="G92" s="5" t="s">
         <x:v>604</x:v>
       </x:c>
-      <x:c r="I92" s="7" t="s">
+      <x:c r="H92" s="5" t="s">
         <x:v>605</x:v>
+      </x:c>
+      <x:c r="I92" s="5" t="s">
+        <x:v>606</x:v>
       </x:c>
       <x:c r="J92">
         <x:v>26</x:v>
@@ -6944,29 +6804,29 @@
       <x:c r="A93">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="B93" s="5" t="s">
-        <x:v>606</x:v>
-      </x:c>
-      <x:c r="C93" s="6">
+      <x:c r="B93" s="3" t="s">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="C93" s="4">
         <x:v>44058</x:v>
       </x:c>
-      <x:c r="D93" s="7" t="s">
-        <x:v>607</x:v>
-      </x:c>
-      <x:c r="E93" s="7" t="s">
+      <x:c r="D93" s="5" t="s">
         <x:v>608</x:v>
       </x:c>
-      <x:c r="F93" s="7" t="s">
+      <x:c r="E93" s="5" t="s">
         <x:v>609</x:v>
       </x:c>
-      <x:c r="G93" s="7" t="s">
+      <x:c r="F93" s="5" t="s">
         <x:v>610</x:v>
       </x:c>
-      <x:c r="H93" s="7" t="s">
+      <x:c r="G93" s="5" t="s">
         <x:v>611</x:v>
       </x:c>
-      <x:c r="I93" s="7" t="s">
+      <x:c r="H93" s="5" t="s">
         <x:v>612</x:v>
+      </x:c>
+      <x:c r="I93" s="5" t="s">
+        <x:v>613</x:v>
       </x:c>
       <x:c r="J93">
         <x:v>10</x:v>
@@ -6985,29 +6845,29 @@
       <x:c r="A94">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="B94" s="5" t="s">
-        <x:v>613</x:v>
-      </x:c>
-      <x:c r="C94" s="6">
+      <x:c r="B94" s="3" t="s">
+        <x:v>614</x:v>
+      </x:c>
+      <x:c r="C94" s="4">
         <x:v>44398</x:v>
       </x:c>
-      <x:c r="D94" s="7" t="s">
-        <x:v>614</x:v>
-      </x:c>
-      <x:c r="E94" s="7" t="s">
+      <x:c r="D94" s="5" t="s">
         <x:v>615</x:v>
       </x:c>
-      <x:c r="F94" s="7" t="s">
+      <x:c r="E94" s="5" t="s">
         <x:v>616</x:v>
       </x:c>
-      <x:c r="G94" s="7" t="s">
+      <x:c r="F94" s="5" t="s">
         <x:v>617</x:v>
       </x:c>
-      <x:c r="H94" s="7" t="s">
+      <x:c r="G94" s="5" t="s">
         <x:v>618</x:v>
       </x:c>
-      <x:c r="I94" s="7" t="s">
+      <x:c r="H94" s="5" t="s">
         <x:v>619</x:v>
+      </x:c>
+      <x:c r="I94" s="5" t="s">
+        <x:v>620</x:v>
       </x:c>
       <x:c r="J94">
         <x:v>11</x:v>
@@ -7018,37 +6878,37 @@
       <x:c r="L94">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M94">
-        <x:v>0</x:v>
+      <x:c r="M94" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="18.75" hidden="1">
       <x:c r="A95">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="B95" s="5" t="s">
-        <x:v>620</x:v>
-      </x:c>
-      <x:c r="C95" s="6">
+      <x:c r="B95" s="3" t="s">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="C95" s="4">
         <x:v>42957</x:v>
       </x:c>
-      <x:c r="D95" s="7" t="s">
-        <x:v>621</x:v>
-      </x:c>
-      <x:c r="E95" s="7" t="s">
+      <x:c r="D95" s="5" t="s">
         <x:v>622</x:v>
       </x:c>
-      <x:c r="F95" s="7" t="s">
+      <x:c r="E95" s="5" t="s">
         <x:v>623</x:v>
       </x:c>
-      <x:c r="G95" s="7" t="s">
+      <x:c r="F95" s="5" t="s">
         <x:v>624</x:v>
       </x:c>
-      <x:c r="H95" s="7" t="s">
+      <x:c r="G95" s="5" t="s">
         <x:v>625</x:v>
       </x:c>
-      <x:c r="I95" s="7" t="s">
+      <x:c r="H95" s="5" t="s">
         <x:v>626</x:v>
+      </x:c>
+      <x:c r="I95" s="5" t="s">
+        <x:v>627</x:v>
       </x:c>
       <x:c r="J95">
         <x:v>12</x:v>
@@ -7067,28 +6927,28 @@
       <x:c r="A96">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="B96" s="5" t="s">
-        <x:v>627</x:v>
-      </x:c>
-      <x:c r="C96" s="6">
+      <x:c r="B96" s="3" t="s">
+        <x:v>628</x:v>
+      </x:c>
+      <x:c r="C96" s="4">
         <x:v>41284</x:v>
       </x:c>
-      <x:c r="D96" s="7" t="s">
+      <x:c r="D96" s="5" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="E96" s="7" t="s">
+      <x:c r="E96" s="5" t="s">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="F96" s="7" t="s">
-        <x:v>568</x:v>
-      </x:c>
-      <x:c r="G96" s="7" t="s">
+      <x:c r="F96" s="5" t="s">
+        <x:v>569</x:v>
+      </x:c>
+      <x:c r="G96" s="5" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="H96" s="7" t="s">
-        <x:v>628</x:v>
-      </x:c>
-      <x:c r="I96" s="7" t="s">
+      <x:c r="H96" s="5" t="s">
+        <x:v>629</x:v>
+      </x:c>
+      <x:c r="I96" s="5" t="s">
         <x:v>130</x:v>
       </x:c>
       <x:c r="J96">
@@ -7108,29 +6968,29 @@
       <x:c r="A97">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="B97" s="5" t="s">
-        <x:v>629</x:v>
-      </x:c>
-      <x:c r="C97" s="6">
+      <x:c r="B97" s="3" t="s">
+        <x:v>630</x:v>
+      </x:c>
+      <x:c r="C97" s="4">
         <x:v>41112</x:v>
       </x:c>
-      <x:c r="D97" s="7" t="s">
-        <x:v>630</x:v>
-      </x:c>
-      <x:c r="E97" s="7" t="s">
+      <x:c r="D97" s="5" t="s">
         <x:v>631</x:v>
       </x:c>
-      <x:c r="F97" s="7" t="s">
+      <x:c r="E97" s="5" t="s">
         <x:v>632</x:v>
       </x:c>
-      <x:c r="G97" s="7" t="s">
+      <x:c r="F97" s="5" t="s">
         <x:v>633</x:v>
       </x:c>
-      <x:c r="H97" s="7" t="s">
+      <x:c r="G97" s="5" t="s">
         <x:v>634</x:v>
       </x:c>
-      <x:c r="I97" s="7" t="s">
+      <x:c r="H97" s="5" t="s">
         <x:v>635</x:v>
+      </x:c>
+      <x:c r="I97" s="5" t="s">
+        <x:v>636</x:v>
       </x:c>
       <x:c r="J97">
         <x:v>34</x:v>
@@ -7149,29 +7009,29 @@
       <x:c r="A98">
         <x:v>97</x:v>
       </x:c>
-      <x:c r="B98" s="5" t="s">
-        <x:v>636</x:v>
-      </x:c>
-      <x:c r="C98" s="6">
+      <x:c r="B98" s="3" t="s">
+        <x:v>637</x:v>
+      </x:c>
+      <x:c r="C98" s="4">
         <x:v>42118</x:v>
       </x:c>
-      <x:c r="D98" s="7" t="s">
-        <x:v>637</x:v>
-      </x:c>
-      <x:c r="E98" s="7" t="s">
+      <x:c r="D98" s="5" t="s">
         <x:v>638</x:v>
       </x:c>
-      <x:c r="F98" s="7" t="s">
+      <x:c r="E98" s="5" t="s">
         <x:v>639</x:v>
       </x:c>
-      <x:c r="G98" s="7" t="s">
+      <x:c r="F98" s="5" t="s">
         <x:v>640</x:v>
       </x:c>
-      <x:c r="H98" s="7" t="s">
+      <x:c r="G98" s="5" t="s">
         <x:v>641</x:v>
       </x:c>
-      <x:c r="I98" s="7" t="s">
+      <x:c r="H98" s="5" t="s">
         <x:v>642</x:v>
+      </x:c>
+      <x:c r="I98" s="5" t="s">
+        <x:v>643</x:v>
       </x:c>
       <x:c r="J98">
         <x:v>9</x:v>
@@ -7190,29 +7050,29 @@
       <x:c r="A99">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="B99" s="5" t="s">
-        <x:v>643</x:v>
-      </x:c>
-      <x:c r="C99" s="6">
+      <x:c r="B99" s="3" t="s">
+        <x:v>644</x:v>
+      </x:c>
+      <x:c r="C99" s="4">
         <x:v>41203</x:v>
       </x:c>
-      <x:c r="D99" s="7" t="s">
-        <x:v>644</x:v>
-      </x:c>
-      <x:c r="E99" s="7" t="s">
+      <x:c r="D99" s="5" t="s">
         <x:v>645</x:v>
       </x:c>
-      <x:c r="F99" s="7" t="s">
+      <x:c r="E99" s="5" t="s">
         <x:v>646</x:v>
       </x:c>
-      <x:c r="G99" s="7" t="s">
+      <x:c r="F99" s="5" t="s">
         <x:v>647</x:v>
       </x:c>
-      <x:c r="H99" s="7" t="s">
+      <x:c r="G99" s="5" t="s">
         <x:v>648</x:v>
       </x:c>
-      <x:c r="I99" s="7" t="s">
+      <x:c r="H99" s="5" t="s">
         <x:v>649</x:v>
+      </x:c>
+      <x:c r="I99" s="5" t="s">
+        <x:v>650</x:v>
       </x:c>
       <x:c r="J99">
         <x:v>18</x:v>
@@ -7231,29 +7091,29 @@
       <x:c r="A100">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="B100" s="5" t="s">
-        <x:v>650</x:v>
-      </x:c>
-      <x:c r="C100" s="6">
+      <x:c r="B100" s="3" t="s">
+        <x:v>651</x:v>
+      </x:c>
+      <x:c r="C100" s="4">
         <x:v>45759</x:v>
       </x:c>
-      <x:c r="D100" s="7" t="s">
-        <x:v>651</x:v>
-      </x:c>
-      <x:c r="E100" s="7" t="s">
+      <x:c r="D100" s="5" t="s">
         <x:v>652</x:v>
       </x:c>
-      <x:c r="F100" s="7" t="s">
+      <x:c r="E100" s="5" t="s">
         <x:v>653</x:v>
       </x:c>
-      <x:c r="G100" s="7" t="s">
-        <x:v>651</x:v>
-      </x:c>
-      <x:c r="H100" s="7" t="s">
+      <x:c r="F100" s="5" t="s">
         <x:v>654</x:v>
       </x:c>
-      <x:c r="I100" s="7" t="s">
+      <x:c r="G100" s="5" t="s">
+        <x:v>652</x:v>
+      </x:c>
+      <x:c r="H100" s="5" t="s">
         <x:v>655</x:v>
+      </x:c>
+      <x:c r="I100" s="5" t="s">
+        <x:v>656</x:v>
       </x:c>
       <x:c r="J100">
         <x:v>5</x:v>
@@ -7268,33 +7128,33 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="101" ht="18.75">
+    <x:row r="101" ht="409.6000061035156">
       <x:c r="A101">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="B101" s="5" t="s">
-        <x:v>656</x:v>
-      </x:c>
-      <x:c r="C101" s="6">
+      <x:c r="B101" s="3" t="s">
+        <x:v>657</x:v>
+      </x:c>
+      <x:c r="C101" s="4">
         <x:v>42971</x:v>
       </x:c>
-      <x:c r="D101" s="7" t="s">
-        <x:v>657</x:v>
-      </x:c>
-      <x:c r="E101" s="7" t="s">
+      <x:c r="D101" s="5" t="s">
         <x:v>658</x:v>
       </x:c>
-      <x:c r="F101" s="7" t="s">
+      <x:c r="E101" s="5" t="s">
         <x:v>659</x:v>
       </x:c>
-      <x:c r="G101" s="7" t="s">
+      <x:c r="F101" s="5" t="s">
         <x:v>660</x:v>
       </x:c>
-      <x:c r="H101" s="7" t="s">
+      <x:c r="G101" s="5" t="s">
         <x:v>661</x:v>
       </x:c>
-      <x:c r="I101" s="7" t="s">
+      <x:c r="H101" s="5" t="s">
         <x:v>662</x:v>
+      </x:c>
+      <x:c r="I101" s="5" t="s">
+        <x:v>663</x:v>
       </x:c>
       <x:c r="J101">
         <x:v>33</x:v>
@@ -7305,37 +7165,37 @@
       <x:c r="L101">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M101">
-        <x:v>1</x:v>
+      <x:c r="M101" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="18.75" hidden="1">
       <x:c r="A102">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="B102" s="5" t="s">
-        <x:v>663</x:v>
-      </x:c>
-      <x:c r="C102" s="6">
+      <x:c r="B102" s="3" t="s">
+        <x:v>664</x:v>
+      </x:c>
+      <x:c r="C102" s="4">
         <x:v>42179</x:v>
       </x:c>
-      <x:c r="D102" s="7" t="s">
-        <x:v>664</x:v>
-      </x:c>
-      <x:c r="E102" s="7" t="s">
+      <x:c r="D102" s="5" t="s">
         <x:v>665</x:v>
       </x:c>
-      <x:c r="F102" s="7" t="s">
+      <x:c r="E102" s="5" t="s">
         <x:v>666</x:v>
       </x:c>
-      <x:c r="G102" s="7" t="s">
+      <x:c r="F102" s="5" t="s">
         <x:v>667</x:v>
       </x:c>
-      <x:c r="H102" s="7" t="s">
+      <x:c r="G102" s="5" t="s">
         <x:v>668</x:v>
       </x:c>
-      <x:c r="I102" s="7" t="s">
+      <x:c r="H102" s="5" t="s">
         <x:v>669</x:v>
+      </x:c>
+      <x:c r="I102" s="5" t="s">
+        <x:v>670</x:v>
       </x:c>
       <x:c r="J102">
         <x:v>15</x:v>
@@ -7354,29 +7214,29 @@
       <x:c r="A103">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="B103" s="5" t="s">
-        <x:v>670</x:v>
-      </x:c>
-      <x:c r="C103" s="6">
+      <x:c r="B103" s="3" t="s">
+        <x:v>671</x:v>
+      </x:c>
+      <x:c r="C103" s="4">
         <x:v>43447</x:v>
       </x:c>
-      <x:c r="D103" s="7" t="s">
-        <x:v>671</x:v>
-      </x:c>
-      <x:c r="E103" s="7" t="s">
+      <x:c r="D103" s="5" t="s">
         <x:v>672</x:v>
       </x:c>
-      <x:c r="F103" s="7" t="s">
+      <x:c r="E103" s="5" t="s">
         <x:v>673</x:v>
       </x:c>
-      <x:c r="G103" s="7" t="s">
+      <x:c r="F103" s="5" t="s">
         <x:v>674</x:v>
       </x:c>
-      <x:c r="H103" s="7" t="s">
+      <x:c r="G103" s="5" t="s">
         <x:v>675</x:v>
       </x:c>
-      <x:c r="I103" s="7" t="s">
+      <x:c r="H103" s="5" t="s">
         <x:v>676</x:v>
+      </x:c>
+      <x:c r="I103" s="5" t="s">
+        <x:v>677</x:v>
       </x:c>
       <x:c r="J103">
         <x:v>5</x:v>
@@ -7395,29 +7255,29 @@
       <x:c r="A104">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="B104" s="5" t="s">
-        <x:v>677</x:v>
-      </x:c>
-      <x:c r="C104" s="6">
+      <x:c r="B104" s="3" t="s">
+        <x:v>678</x:v>
+      </x:c>
+      <x:c r="C104" s="4">
         <x:v>42461</x:v>
       </x:c>
-      <x:c r="D104" s="7" t="s">
-        <x:v>678</x:v>
-      </x:c>
-      <x:c r="E104" s="7" t="s">
+      <x:c r="D104" s="5" t="s">
         <x:v>679</x:v>
       </x:c>
-      <x:c r="F104" s="7" t="s">
+      <x:c r="E104" s="5" t="s">
         <x:v>680</x:v>
       </x:c>
-      <x:c r="G104" s="7" t="s">
+      <x:c r="F104" s="5" t="s">
         <x:v>681</x:v>
       </x:c>
-      <x:c r="H104" s="7" t="s">
+      <x:c r="G104" s="5" t="s">
         <x:v>682</x:v>
       </x:c>
-      <x:c r="I104" s="7" t="s">
+      <x:c r="H104" s="5" t="s">
         <x:v>683</x:v>
+      </x:c>
+      <x:c r="I104" s="5" t="s">
+        <x:v>684</x:v>
       </x:c>
       <x:c r="J104">
         <x:v>55</x:v>
@@ -7432,33 +7292,33 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="105" ht="18.75">
+    <x:row r="105" ht="409.6000061035156">
       <x:c r="A105">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="B105" s="5" t="s">
-        <x:v>684</x:v>
-      </x:c>
-      <x:c r="C105" s="6">
+      <x:c r="B105" s="3" t="s">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="C105" s="4">
         <x:v>43901</x:v>
       </x:c>
-      <x:c r="D105" s="7" t="s">
-        <x:v>685</x:v>
-      </x:c>
-      <x:c r="E105" s="7" t="s">
+      <x:c r="D105" s="5" t="s">
         <x:v>686</x:v>
       </x:c>
-      <x:c r="F105" s="7" t="s">
+      <x:c r="E105" s="5" t="s">
         <x:v>687</x:v>
       </x:c>
-      <x:c r="G105" s="7" t="s">
+      <x:c r="F105" s="5" t="s">
         <x:v>688</x:v>
       </x:c>
-      <x:c r="H105" s="7" t="s">
+      <x:c r="G105" s="5" t="s">
         <x:v>689</x:v>
       </x:c>
-      <x:c r="I105" s="7" t="s">
+      <x:c r="H105" s="5" t="s">
         <x:v>690</x:v>
+      </x:c>
+      <x:c r="I105" s="5" t="s">
+        <x:v>691</x:v>
       </x:c>
       <x:c r="J105">
         <x:v>7</x:v>
@@ -7474,7 +7334,7 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A$1:M$1048576">
+  <x:conditionalFormatting sqref="A1:M1048576">
     <x:cfRule type="expression" dxfId="0" priority="1">
       <x:formula>MOD(ROW(),2)=1</x:formula>
     </x:cfRule>

</xml_diff>